<commit_message>
Sync Tracker with spend log (5 added, 0 updated, 0 removed)
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="329">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -900,6 +900,9 @@
     <t xml:space="preserve">Paid so far</t>
   </si>
   <si>
+    <t xml:space="preserve">Log ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">28/09/2026</t>
   </si>
   <si>
@@ -982,6 +985,33 @@
   </si>
   <si>
     <t xml:space="preserve">Dinner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMoney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfx8jx3909u</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfx90yw8xl4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfx9bgghgpi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">20/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kimbap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfusx39nkux</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eggs and Sparkling water</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfutaqk8eyk</t>
   </si>
 </sst>
 </file>
@@ -1737,11 +1767,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>53.96</v>
+        <v>80.82</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">D7+D13-F7</f>
-        <v>1167.04</v>
+        <v>1140.18</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2031,11 +2061,11 @@
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
-        <v>17.96</v>
+        <v>41.87</v>
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3372.04</v>
+        <v>3348.13</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
@@ -2052,11 +2082,11 @@
       </c>
       <c r="C23" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A23)</f>
-        <v>0</v>
+        <v>2.95</v>
       </c>
       <c r="D23" s="18" t="n">
         <f aca="false">B23-C23</f>
-        <v>970</v>
+        <v>967.05</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B23/$B$3)</f>
@@ -2136,11 +2166,11 @@
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">SUM(C20:C26)</f>
-        <v>2728.46</v>
+        <v>2755.32</v>
       </c>
       <c r="D27" s="24" t="n">
         <f aca="false">SUM(D20:D26)</f>
-        <v>7271.54</v>
+        <v>7244.68</v>
       </c>
       <c r="E27" s="25" t="n">
         <f aca="false">SUM(E20:E26)</f>
@@ -2164,7 +2194,7 @@
       </c>
       <c r="B31" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2728.46</v>
+        <v>2755.32</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2182,7 +2212,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7271.54</v>
+        <v>7244.68</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2190,12 +2220,12 @@
         <v>44</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="20" t="s">
         <v>46</v>
       </c>
@@ -2203,25 +2233,25 @@
         <v>8034.27</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
         <v>47</v>
       </c>
       <c r="B39" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2728.46</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>2755.32</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
         <v>48</v>
       </c>
       <c r="B40" s="27" t="n">
         <f aca="false">B38-B39</f>
-        <v>5305.81</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5278.95</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="20" t="s">
         <v>49</v>
       </c>
@@ -2230,7 +2260,7 @@
         <v>1965.73</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="20" t="s">
         <v>50</v>
       </c>
@@ -3325,7 +3355,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
         <v>27</v>
       </c>
@@ -4283,7 +4313,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="42" t="s">
         <v>27</v>
       </c>
@@ -4329,7 +4359,7 @@
         <v>1397.02</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>163</v>
       </c>
@@ -5294,7 +5324,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:J1000"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -5306,6 +5336,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5342,21 +5373,24 @@
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2728.46</v>
+        <v>2755.32</v>
+      </c>
+      <c r="J4" s="7" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C5" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="51" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="E5" s="52" t="n">
         <v>667.6</v>
@@ -5374,16 +5408,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C6" s="51" t="s">
         <v>38</v>
       </c>
       <c r="D6" s="51" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E6" s="52" t="n">
         <v>281.62</v>
@@ -5392,16 +5426,16 @@
         <v>41</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2728.46</v>
+        <v>2755.32</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B7" s="51" t="s">
         <v>11</v>
@@ -5410,7 +5444,7 @@
         <v>34</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E7" s="52" t="n">
         <v>36</v>
@@ -5419,25 +5453,25 @@
         <v>41</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7271.54</v>
+        <v>7244.68</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C8" s="51" t="s">
         <v>38</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E8" s="52" t="n">
         <v>19</v>
@@ -5448,16 +5482,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C9" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D9" s="51" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E9" s="52" t="n">
         <v>87.7</v>
@@ -5468,7 +5502,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B10" s="51" t="s">
         <v>13</v>
@@ -5477,7 +5511,7 @@
         <v>34</v>
       </c>
       <c r="D10" s="51" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E10" s="52" t="n">
         <v>239.55</v>
@@ -5488,7 +5522,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B11" s="51" t="s">
         <v>13</v>
@@ -5497,7 +5531,7 @@
         <v>34</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E11" s="52" t="n">
         <v>52.24</v>
@@ -5508,16 +5542,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C12" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E12" s="52" t="n">
         <v>211.52</v>
@@ -5528,7 +5562,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B13" s="51" t="s">
         <v>13</v>
@@ -5537,7 +5571,7 @@
         <v>34</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E13" s="52" t="n">
         <v>137.26</v>
@@ -5548,7 +5582,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B14" s="51" t="s">
         <v>13</v>
@@ -5557,7 +5591,7 @@
         <v>34</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E14" s="52" t="n">
         <v>338.05</v>
@@ -5568,7 +5602,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B15" s="51" t="s">
         <v>13</v>
@@ -5577,7 +5611,7 @@
         <v>34</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E15" s="52" t="n">
         <v>66.78</v>
@@ -5588,7 +5622,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="51" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B16" s="51" t="s">
         <v>13</v>
@@ -5597,7 +5631,7 @@
         <v>34</v>
       </c>
       <c r="D16" s="51" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E16" s="52" t="n">
         <v>300.97</v>
@@ -5608,7 +5642,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="51" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B17" s="51" t="s">
         <v>13</v>
@@ -5617,7 +5651,7 @@
         <v>34</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E17" s="52" t="n">
         <v>226.17</v>
@@ -5628,10 +5662,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="51" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C18" s="51" t="s">
         <v>38</v>
@@ -5648,16 +5682,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="51" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="C19" s="51" t="s">
         <v>38</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E19" s="52" t="n">
         <v>32.4</v>
@@ -5668,7 +5702,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="51" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B20" s="51" t="s">
         <v>11</v>
@@ -5677,7 +5711,7 @@
         <v>35</v>
       </c>
       <c r="D20" s="51" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E20" s="52" t="n">
         <v>3.05</v>
@@ -5688,7 +5722,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="51" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B21" s="51" t="s">
         <v>11</v>
@@ -5697,7 +5731,7 @@
         <v>35</v>
       </c>
       <c r="D21" s="51" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E21" s="52" t="n">
         <v>14.91</v>
@@ -5707,44 +5741,119 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="51"/>
-      <c r="B22" s="51"/>
-      <c r="C22" s="51"/>
-      <c r="D22" s="51"/>
-      <c r="E22" s="52"/>
-      <c r="F22" s="51"/>
+      <c r="A22" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="B22" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="51" t="s">
+        <v>320</v>
+      </c>
+      <c r="E22" s="52" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="F22" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J22" s="0" t="s">
+        <v>321</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="51"/>
-      <c r="B23" s="51"/>
-      <c r="C23" s="51"/>
-      <c r="D23" s="51"/>
-      <c r="E23" s="52"/>
-      <c r="F23" s="51"/>
+      <c r="A23" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="B23" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="51" t="s">
+        <v>318</v>
+      </c>
+      <c r="E23" s="52" t="n">
+        <v>3.05</v>
+      </c>
+      <c r="F23" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J23" s="0" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="51"/>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="52"/>
-      <c r="F24" s="51"/>
+      <c r="A24" s="51" t="s">
+        <v>316</v>
+      </c>
+      <c r="B24" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D24" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="E24" s="52" t="n">
+        <v>14.91</v>
+      </c>
+      <c r="F24" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J24" s="0" t="s">
+        <v>323</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="51"/>
-      <c r="B25" s="51"/>
-      <c r="C25" s="51"/>
-      <c r="D25" s="51"/>
-      <c r="E25" s="52"/>
-      <c r="F25" s="51"/>
+      <c r="A25" s="51" t="s">
+        <v>324</v>
+      </c>
+      <c r="B25" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D25" s="51" t="s">
+        <v>325</v>
+      </c>
+      <c r="E25" s="52" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F25" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J25" s="0" t="s">
+        <v>326</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="51"/>
-      <c r="B26" s="51"/>
-      <c r="C26" s="51"/>
-      <c r="D26" s="51"/>
-      <c r="E26" s="52"/>
-      <c r="F26" s="51"/>
+      <c r="A26" s="51" t="s">
+        <v>324</v>
+      </c>
+      <c r="B26" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D26" s="51" t="s">
+        <v>327</v>
+      </c>
+      <c r="E26" s="52" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="F26" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J26" s="0" t="s">
+        <v>328</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="51"/>

</xml_diff>

<commit_message>
Sync Tracker with spend log (1 added, 0 updated, 0 removed)
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="330">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -1012,6 +1012,9 @@
   </si>
   <si>
     <t xml:space="preserve">mvfutaqk8eyk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvg586qrpc9q</t>
   </si>
 </sst>
 </file>
@@ -1767,11 +1770,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>80.82</v>
+        <v>86.72</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">D7+D13-F7</f>
-        <v>1140.18</v>
+        <v>1134.28</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2082,11 +2085,11 @@
       </c>
       <c r="C23" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A23)</f>
-        <v>2.95</v>
+        <v>8.85</v>
       </c>
       <c r="D23" s="18" t="n">
         <f aca="false">B23-C23</f>
-        <v>967.05</v>
+        <v>961.15</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B23/$B$3)</f>
@@ -2166,11 +2169,11 @@
       </c>
       <c r="C27" s="24" t="n">
         <f aca="false">SUM(C20:C26)</f>
-        <v>2755.32</v>
+        <v>2761.22</v>
       </c>
       <c r="D27" s="24" t="n">
         <f aca="false">SUM(D20:D26)</f>
-        <v>7244.68</v>
+        <v>7238.78</v>
       </c>
       <c r="E27" s="25" t="n">
         <f aca="false">SUM(E20:E26)</f>
@@ -2194,7 +2197,7 @@
       </c>
       <c r="B31" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2755.32</v>
+        <v>2761.22</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2212,7 +2215,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7244.68</v>
+        <v>7238.78</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2239,7 +2242,7 @@
       </c>
       <c r="B39" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2755.32</v>
+        <v>2761.22</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2248,7 +2251,7 @@
       </c>
       <c r="B40" s="27" t="n">
         <f aca="false">B38-B39</f>
-        <v>5278.95</v>
+        <v>5273.05</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5336,7 +5339,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="10" min="10" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5373,7 +5376,7 @@
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2755.32</v>
+        <v>2761.22</v>
       </c>
       <c r="J4" s="7" t="s">
         <v>291</v>
@@ -5430,7 +5433,7 @@
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2755.32</v>
+        <v>2761.22</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5457,7 +5460,7 @@
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7244.68</v>
+        <v>7238.78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5759,7 +5762,7 @@
       <c r="F22" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J22" s="0" t="s">
+      <c r="J22" s="1" t="s">
         <v>321</v>
       </c>
     </row>
@@ -5782,7 +5785,7 @@
       <c r="F23" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J23" s="0" t="s">
+      <c r="J23" s="1" t="s">
         <v>322</v>
       </c>
     </row>
@@ -5805,7 +5808,7 @@
       <c r="F24" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J24" s="0" t="s">
+      <c r="J24" s="1" t="s">
         <v>323</v>
       </c>
     </row>
@@ -5828,7 +5831,7 @@
       <c r="F25" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J25" s="0" t="s">
+      <c r="J25" s="1" t="s">
         <v>326</v>
       </c>
     </row>
@@ -5851,17 +5854,32 @@
       <c r="F26" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J26" s="0" t="s">
+      <c r="J26" s="1" t="s">
         <v>328</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="51"/>
-      <c r="B27" s="51"/>
-      <c r="C27" s="51"/>
-      <c r="D27" s="51"/>
-      <c r="E27" s="52"/>
-      <c r="F27" s="51"/>
+      <c r="A27" s="51" t="s">
+        <v>324</v>
+      </c>
+      <c r="B27" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="51" t="s">
+        <v>320</v>
+      </c>
+      <c r="E27" s="52" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F27" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>329</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="51"/>

</xml_diff>

<commit_message>
Daily log categories match Budget lines; add Shopping & misc
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="339">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Ground costs only (accommodation, food, local transport, activities). Korea &amp; Japan appear twice – spend is combined on their first row.</t>
+    <t xml:space="preserve">Ground costs only (accommodation, food, local transport, activities, shopping &amp; misc). Korea &amp; Japan appear twice – spend is combined on their first row.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Budget by category</t>
@@ -141,6 +141,9 @@
     <t xml:space="preserve">Activities</t>
   </si>
   <si>
+    <t xml:space="preserve">Shopping &amp; misc</t>
+  </si>
+  <si>
     <t xml:space="preserve">Insurance &amp; admin</t>
   </si>
   <si>
@@ -219,6 +222,9 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
+    <t xml:space="preserve">Shopping &amp; misc (£)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Incheon – Incheon Airport Hotel Seattle</t>
   </si>
   <si>
@@ -981,18 +987,15 @@
     <t xml:space="preserve">eSIM #1 – 50GB, 45 days</t>
   </si>
   <si>
+    <t xml:space="preserve">TMoney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvfx8jx3909u</t>
+  </si>
+  <si>
     <t xml:space="preserve">Coffee</t>
   </si>
   <si>
-    <t xml:space="preserve">Dinner</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TMoney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mvfx8jx3909u</t>
-  </si>
-  <si>
     <t xml:space="preserve">mvfx90yw8xl4</t>
   </si>
   <si>
@@ -1039,15 +1042,6 @@
   </si>
   <si>
     <t xml:space="preserve">mvgm1pq2sx7l</t>
-  </si>
-  <si>
-    <t xml:space="preserve">21/10/2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mvha28vt2umu</t>
   </si>
 </sst>
 </file>
@@ -1724,7 +1718,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
@@ -1795,19 +1789,19 @@
       </c>
       <c r="D7" s="10" t="n">
         <f aca="false">SUM(Itinerary!K5:K6)</f>
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="E7" s="11" t="n">
         <f aca="false">IF(C7=0,0,D7/C7)</f>
-        <v>60.3333333333333</v>
+        <v>65.3333333333333</v>
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>113.73</v>
+        <v>91.51</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">D7+D13-F7</f>
-        <v>1107.27</v>
+        <v>1244.49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1823,11 +1817,11 @@
       </c>
       <c r="D8" s="10" t="n">
         <f aca="false">SUM(Itinerary!K7:K11)</f>
-        <v>2766.02</v>
+        <v>2866.02</v>
       </c>
       <c r="E8" s="11" t="n">
         <f aca="false">IF(C8=0,0,D8/C8)</f>
-        <v>138.301</v>
+        <v>143.301</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1835,7 +1829,7 @@
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">D8+D14-F8</f>
-        <v>3484</v>
+        <v>3659</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1851,11 +1845,11 @@
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUM(Itinerary!K12:K13)</f>
-        <v>535</v>
+        <v>575</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">IF(C9=0,0,D9/C9)</f>
-        <v>66.875</v>
+        <v>71.875</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1863,7 +1857,7 @@
       </c>
       <c r="G9" s="12" t="n">
         <f aca="false">D9-F9</f>
-        <v>535</v>
+        <v>575</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1879,11 +1873,11 @@
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">SUM(Itinerary!K14:K15)</f>
-        <v>700</v>
+        <v>735</v>
       </c>
       <c r="E10" s="11" t="n">
         <f aca="false">IF(C10=0,0,D10/C10)</f>
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1891,7 +1885,7 @@
       </c>
       <c r="G10" s="12" t="n">
         <f aca="false">D10-F10</f>
-        <v>700</v>
+        <v>735</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1907,11 +1901,11 @@
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">SUM(Itinerary!K16:K17)</f>
-        <v>696</v>
+        <v>736</v>
       </c>
       <c r="E11" s="11" t="n">
         <f aca="false">IF(C11=0,0,D11/C11)</f>
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1919,7 +1913,7 @@
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">D11-F11</f>
-        <v>696</v>
+        <v>736</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1935,11 +1929,11 @@
       </c>
       <c r="D12" s="10" t="n">
         <f aca="false">SUM(Itinerary!K18:K19)</f>
-        <v>1195</v>
+        <v>1245</v>
       </c>
       <c r="E12" s="11" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>119.5</v>
+        <v>124.5</v>
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1947,7 +1941,7 @@
       </c>
       <c r="G12" s="12" t="n">
         <f aca="false">D12-F12</f>
-        <v>1195</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1963,11 +1957,11 @@
       </c>
       <c r="D13" s="10" t="n">
         <f aca="false">SUM(Itinerary!K20:K20)</f>
-        <v>1040</v>
+        <v>1140</v>
       </c>
       <c r="E13" s="11" t="n">
         <f aca="false">IF(C13=0,0,D13/C13)</f>
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F13" s="13" t="s">
         <v>24</v>
@@ -1987,11 +1981,11 @@
       </c>
       <c r="D14" s="10" t="n">
         <f aca="false">SUM(Itinerary!K21:K24)</f>
-        <v>2079</v>
+        <v>2154</v>
       </c>
       <c r="E14" s="11" t="n">
         <f aca="false">IF(C14=0,0,D14/C14)</f>
-        <v>138.6</v>
+        <v>143.6</v>
       </c>
       <c r="F14" s="13" t="s">
         <v>26</v>
@@ -2009,11 +2003,11 @@
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">SUM(D7:D14)</f>
-        <v>9192.02</v>
+        <v>9647.02</v>
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">IF(C15=0,0,D15/C15)</f>
-        <v>101.011208791209</v>
+        <v>106.011208791209</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="15"/>
@@ -2097,11 +2091,11 @@
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
-        <v>65.48</v>
+        <v>43.26</v>
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3324.52</v>
+        <v>3346.74</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
@@ -2139,11 +2133,11 @@
       </c>
       <c r="C24" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A24)</f>
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="D24" s="18" t="n">
         <f aca="false">B24-C24</f>
-        <v>1026.6</v>
+        <v>1030</v>
       </c>
       <c r="E24" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B24/$B$3)</f>
@@ -2155,127 +2149,142 @@
         <v>38</v>
       </c>
       <c r="B25" s="17" t="n">
+        <f aca="false">Itinerary!O25</f>
+        <v>455</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A25)</f>
+        <v>3.4</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <f aca="false">B25-C25</f>
+        <v>451.6</v>
+      </c>
+      <c r="E25" s="19" t="n">
+        <f aca="false">IF($B$3=0,0,B25/$B$3)</f>
+        <v>0.0455</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="B26" s="17" t="n">
         <f aca="false">'Admin &amp; checklist'!B9</f>
         <v>457.66</v>
       </c>
-      <c r="C25" s="18" t="n">
-        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A25)</f>
+      <c r="C26" s="18" t="n">
+        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A26)</f>
         <v>346.66</v>
       </c>
-      <c r="D25" s="18" t="n">
-        <f aca="false">B25-C25</f>
+      <c r="D26" s="18" t="n">
+        <f aca="false">B26-C26</f>
         <v>111</v>
       </c>
-      <c r="E25" s="19" t="n">
-        <f aca="false">IF($B$3=0,0,B25/$B$3)</f>
+      <c r="E26" s="19" t="n">
+        <f aca="false">IF($B$3=0,0,B26/$B$3)</f>
         <v>0.045766</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26" s="21" t="n">
-        <f aca="false">$B$3-SUM(B20:B25)</f>
-        <v>-1356.5</v>
-      </c>
-      <c r="C26" s="22" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="21" t="n">
+        <f aca="false">$B$3-SUM(B20:B26)</f>
+        <v>-1811.5</v>
+      </c>
+      <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,"Other")</f>
         <v>0</v>
       </c>
-      <c r="D26" s="22" t="n">
-        <f aca="false">B26-C26</f>
-        <v>-1356.5</v>
-      </c>
-      <c r="E26" s="23" t="n">
-        <f aca="false">IF($B$3=0,0,B26/$B$3)</f>
-        <v>-0.13565</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="s">
+      <c r="D27" s="22" t="n">
+        <f aca="false">B27-C27</f>
+        <v>-1811.5</v>
+      </c>
+      <c r="E27" s="23" t="n">
+        <f aca="false">IF($B$3=0,0,B27/$B$3)</f>
+        <v>-0.18115</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B27" s="24" t="n">
-        <f aca="false">SUM(B20:B26)</f>
+      <c r="B28" s="24" t="n">
+        <f aca="false">SUM(B20:B27)</f>
         <v>10000</v>
       </c>
-      <c r="C27" s="24" t="n">
-        <f aca="false">SUM(C20:C26)</f>
-        <v>2788.23</v>
-      </c>
-      <c r="D27" s="24" t="n">
-        <f aca="false">SUM(D20:D26)</f>
-        <v>7211.77</v>
-      </c>
-      <c r="E27" s="25" t="n">
-        <f aca="false">SUM(E20:E26)</f>
+      <c r="C28" s="24" t="n">
+        <f aca="false">SUM(C20:C27)</f>
+        <v>2766.01</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <f aca="false">SUM(D20:D27)</f>
+        <v>7233.99</v>
+      </c>
+      <c r="E28" s="25" t="n">
+        <f aca="false">SUM(E20:E27)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="26" t="str">
-        <f aca="false">IF(B26&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B26,"£#,##0"),IF(B26&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
-        <v>⚠ Plan is over budget by £1,357</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="s">
-        <v>40</v>
-      </c>
-    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="26" t="str">
+        <f aca="false">IF(B27&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B27,"£#,##0"),IF(B27&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
+        <v>⚠ Plan is over budget by £1,812</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="B31" s="27" t="n">
-        <f aca="false">Tracker!I4</f>
-        <v>2788.23</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="22" t="n">
-        <f aca="false">Tracker!I5</f>
-        <v>0</v>
+      <c r="B32" s="27" t="n">
+        <f aca="false">Tracker!I4</f>
+        <v>2766.01</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="27" t="n">
+      <c r="B33" s="22" t="n">
+        <f aca="false">Tracker!I5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7211.77</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="s">
+        <v>7233.99</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
         <v>45</v>
       </c>
     </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20" t="s">
+      <c r="A38" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="B38" s="28" t="n">
-        <v>8034.27</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="20" t="s">
         <v>47</v>
       </c>
-      <c r="B39" s="27" t="n">
-        <f aca="false">Tracker!I4</f>
-        <v>2788.23</v>
+      <c r="B39" s="28" t="n">
+        <v>8034.27</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2283,8 +2292,8 @@
         <v>48</v>
       </c>
       <c r="B40" s="27" t="n">
-        <f aca="false">B38-B39</f>
-        <v>5246.04</v>
+        <f aca="false">Tracker!I4</f>
+        <v>2766.01</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2292,8 +2301,8 @@
         <v>49</v>
       </c>
       <c r="B41" s="27" t="n">
-        <f aca="false">MAX(0,B3-B38)</f>
-        <v>1965.73</v>
+        <f aca="false">B39-B40</f>
+        <v>5268.26</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2301,8 +2310,17 @@
         <v>50</v>
       </c>
       <c r="B42" s="27" t="n">
-        <f aca="false">MAX(0,SUM(B20:B25)-B38)</f>
-        <v>3322.23</v>
+        <f aca="false">MAX(0,B3-B39)</f>
+        <v>1965.73</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" s="27" t="n">
+        <f aca="false">MAX(0,SUM(B20:B26)-B39)</f>
+        <v>3777.23</v>
       </c>
     </row>
   </sheetData>
@@ -2321,7 +2339,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
@@ -2335,16 +2353,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2352,7 +2371,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>5</v>
@@ -2361,34 +2380,37 @@
         <v>6</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
+      </c>
+      <c r="O4" s="7" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2396,10 +2418,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D5" s="29" t="n">
         <v>1</v>
@@ -2426,19 +2448,22 @@
         <v>15</v>
       </c>
       <c r="K5" s="12" t="n">
-        <f aca="false">G5+H5+I5+J5</f>
-        <v>66</v>
+        <f aca="false">G5+H5+I5+J5+O5</f>
+        <v>71</v>
       </c>
       <c r="L5" s="12" t="n">
         <f aca="false">IF(D5=0,0,K5/D5)</f>
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="M5" s="9" t="str">
         <f aca="false">IF(Hotels!G5="Booked","Yes",IF(Hotels!G5="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N5" s="31" t="s">
-        <v>66</v>
+        <v>68</v>
+      </c>
+      <c r="O5" s="30" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2446,10 +2471,10 @@
         <v>11</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D6" s="29" t="n">
         <v>2</v>
@@ -2476,19 +2501,22 @@
         <v>60</v>
       </c>
       <c r="K6" s="12" t="n">
-        <f aca="false">G6+H6+I6+J6</f>
-        <v>115</v>
+        <f aca="false">G6+H6+I6+J6+O6</f>
+        <v>125</v>
       </c>
       <c r="L6" s="12" t="n">
         <f aca="false">IF(D6=0,0,K6/D6)</f>
-        <v>57.5</v>
+        <v>62.5</v>
       </c>
       <c r="M6" s="9" t="str">
         <f aca="false">IF(Hotels!G6="Booked","Yes",IF(Hotels!G6="Staying with friends","N/A – host","No"))</f>
         <v>N/A – host</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>69</v>
+        <v>71</v>
+      </c>
+      <c r="O6" s="30" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2496,10 +2524,10 @@
         <v>13</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D7" s="29" t="n">
         <v>3</v>
@@ -2526,19 +2554,22 @@
         <v>114</v>
       </c>
       <c r="K7" s="12" t="n">
-        <f aca="false">G7+H7+I7+J7</f>
-        <v>475.79</v>
+        <f aca="false">G7+H7+I7+J7+O7</f>
+        <v>490.79</v>
       </c>
       <c r="L7" s="12" t="n">
         <f aca="false">IF(D7=0,0,K7/D7)</f>
-        <v>158.596666666667</v>
+        <v>163.596666666667</v>
       </c>
       <c r="M7" s="9" t="str">
         <f aca="false">IF(Hotels!G7="Booked","Yes",IF(Hotels!G7="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N7" s="31" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="O7" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2546,10 +2577,10 @@
         <v>13</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D8" s="29" t="n">
         <v>3</v>
@@ -2576,19 +2607,22 @@
         <v>114</v>
       </c>
       <c r="K8" s="12" t="n">
-        <f aca="false">G8+H8+I8+J8</f>
-        <v>413.04</v>
+        <f aca="false">G8+H8+I8+J8+O8</f>
+        <v>428.04</v>
       </c>
       <c r="L8" s="12" t="n">
         <f aca="false">IF(D8=0,0,K8/D8)</f>
-        <v>137.68</v>
+        <v>142.68</v>
       </c>
       <c r="M8" s="9" t="str">
         <f aca="false">IF(Hotels!G8="Booked","Yes",IF(Hotels!G8="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N8" s="31" t="s">
-        <v>75</v>
+        <v>77</v>
+      </c>
+      <c r="O8" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2596,10 +2630,10 @@
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D9" s="29" t="n">
         <v>5</v>
@@ -2626,19 +2660,22 @@
         <v>190</v>
       </c>
       <c r="K9" s="12" t="n">
-        <f aca="false">G9+H9+I9+J9</f>
-        <v>663.05</v>
+        <f aca="false">G9+H9+I9+J9+O9</f>
+        <v>688.05</v>
       </c>
       <c r="L9" s="12" t="n">
         <f aca="false">IF(D9=0,0,K9/D9)</f>
-        <v>132.61</v>
+        <v>137.61</v>
       </c>
       <c r="M9" s="9" t="str">
         <f aca="false">IF(Hotels!G9="Booked","Yes",IF(Hotels!G9="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N9" s="31" t="s">
-        <v>78</v>
+        <v>80</v>
+      </c>
+      <c r="O9" s="30" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2646,10 +2683,10 @@
         <v>13</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D10" s="29" t="n">
         <v>3</v>
@@ -2676,19 +2713,22 @@
         <v>114</v>
       </c>
       <c r="K10" s="12" t="n">
-        <f aca="false">G10+H10+I10+J10</f>
-        <v>425.17</v>
+        <f aca="false">G10+H10+I10+J10+O10</f>
+        <v>440.17</v>
       </c>
       <c r="L10" s="12" t="n">
         <f aca="false">IF(D10=0,0,K10/D10)</f>
-        <v>141.723333333333</v>
+        <v>146.723333333333</v>
       </c>
       <c r="M10" s="9" t="str">
         <f aca="false">IF(Hotels!G10="Booked","Yes",IF(Hotels!G10="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N10" s="31" t="s">
-        <v>81</v>
+        <v>83</v>
+      </c>
+      <c r="O10" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2696,10 +2736,10 @@
         <v>13</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D11" s="29" t="n">
         <v>6</v>
@@ -2726,19 +2766,22 @@
         <v>348</v>
       </c>
       <c r="K11" s="12" t="n">
-        <f aca="false">G11+H11+I11+J11</f>
-        <v>788.97</v>
+        <f aca="false">G11+H11+I11+J11+O11</f>
+        <v>818.97</v>
       </c>
       <c r="L11" s="12" t="n">
         <f aca="false">IF(D11=0,0,K11/D11)</f>
-        <v>131.495</v>
+        <v>136.495</v>
       </c>
       <c r="M11" s="9" t="str">
         <f aca="false">IF(Hotels!G11="Booked","Yes",IF(Hotels!G11="Staying with friends","N/A – host","No"))</f>
         <v>Yes</v>
       </c>
       <c r="N11" s="31" t="s">
-        <v>84</v>
+        <v>86</v>
+      </c>
+      <c r="O11" s="30" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2746,10 +2789,10 @@
         <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D12" s="29" t="n">
         <v>3</v>
@@ -2776,19 +2819,22 @@
         <v>45</v>
       </c>
       <c r="K12" s="12" t="n">
-        <f aca="false">G12+H12+I12+J12</f>
-        <v>190</v>
+        <f aca="false">G12+H12+I12+J12+O12</f>
+        <v>205</v>
       </c>
       <c r="L12" s="12" t="n">
         <f aca="false">IF(D12=0,0,K12/D12)</f>
-        <v>63.3333333333333</v>
+        <v>68.3333333333333</v>
       </c>
       <c r="M12" s="9" t="str">
         <f aca="false">IF(Hotels!G12="Booked","Yes",IF(Hotels!G12="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N12" s="31" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="O12" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2796,10 +2842,10 @@
         <v>15</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D13" s="29" t="n">
         <v>5</v>
@@ -2826,19 +2872,22 @@
         <v>135</v>
       </c>
       <c r="K13" s="12" t="n">
-        <f aca="false">G13+H13+I13+J13</f>
-        <v>345</v>
+        <f aca="false">G13+H13+I13+J13+O13</f>
+        <v>370</v>
       </c>
       <c r="L13" s="12" t="n">
         <f aca="false">IF(D13=0,0,K13/D13)</f>
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="M13" s="9" t="str">
         <f aca="false">IF(Hotels!G13="Booked","Yes",IF(Hotels!G13="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N13" s="31" t="s">
-        <v>90</v>
+        <v>92</v>
+      </c>
+      <c r="O13" s="30" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2846,10 +2895,10 @@
         <v>17</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D14" s="29" t="n">
         <v>4</v>
@@ -2876,19 +2925,22 @@
         <v>190</v>
       </c>
       <c r="K14" s="12" t="n">
-        <f aca="false">G14+H14+I14+J14</f>
-        <v>440</v>
+        <f aca="false">G14+H14+I14+J14+O14</f>
+        <v>460</v>
       </c>
       <c r="L14" s="12" t="n">
         <f aca="false">IF(D14=0,0,K14/D14)</f>
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="M14" s="9" t="str">
         <f aca="false">IF(Hotels!G14="Booked","Yes",IF(Hotels!G14="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N14" s="31" t="s">
-        <v>93</v>
+        <v>95</v>
+      </c>
+      <c r="O14" s="30" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2896,10 +2948,10 @@
         <v>17</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D15" s="29" t="n">
         <v>3</v>
@@ -2926,19 +2978,22 @@
         <v>75</v>
       </c>
       <c r="K15" s="12" t="n">
-        <f aca="false">G15+H15+I15+J15</f>
-        <v>260</v>
+        <f aca="false">G15+H15+I15+J15+O15</f>
+        <v>275</v>
       </c>
       <c r="L15" s="12" t="n">
         <f aca="false">IF(D15=0,0,K15/D15)</f>
-        <v>86.6666666666667</v>
+        <v>91.6666666666667</v>
       </c>
       <c r="M15" s="9" t="str">
         <f aca="false">IF(Hotels!G15="Booked","Yes",IF(Hotels!G15="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N15" s="31" t="s">
-        <v>96</v>
+        <v>98</v>
+      </c>
+      <c r="O15" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2946,10 +3001,10 @@
         <v>19</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D16" s="29" t="n">
         <v>3</v>
@@ -2976,19 +3031,22 @@
         <v>66</v>
       </c>
       <c r="K16" s="12" t="n">
-        <f aca="false">G16+H16+I16+J16</f>
-        <v>231</v>
+        <f aca="false">G16+H16+I16+J16+O16</f>
+        <v>246</v>
       </c>
       <c r="L16" s="12" t="n">
         <f aca="false">IF(D16=0,0,K16/D16)</f>
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="M16" s="9" t="str">
         <f aca="false">IF(Hotels!G16="Booked","Yes",IF(Hotels!G16="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N16" s="31" t="s">
-        <v>99</v>
+        <v>101</v>
+      </c>
+      <c r="O16" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2996,10 +3054,10 @@
         <v>19</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D17" s="29" t="n">
         <v>5</v>
@@ -3026,19 +3084,22 @@
         <v>200</v>
       </c>
       <c r="K17" s="12" t="n">
-        <f aca="false">G17+H17+I17+J17</f>
-        <v>465</v>
+        <f aca="false">G17+H17+I17+J17+O17</f>
+        <v>490</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">IF(D17=0,0,K17/D17)</f>
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="M17" s="9" t="str">
         <f aca="false">IF(Hotels!G17="Booked","Yes",IF(Hotels!G17="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N17" s="31" t="s">
-        <v>102</v>
+        <v>104</v>
+      </c>
+      <c r="O17" s="30" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3046,10 +3107,10 @@
         <v>21</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="D18" s="29" t="n">
         <v>6</v>
@@ -3076,19 +3137,22 @@
         <v>270</v>
       </c>
       <c r="K18" s="12" t="n">
-        <f aca="false">G18+H18+I18+J18</f>
-        <v>890</v>
+        <f aca="false">G18+H18+I18+J18+O18</f>
+        <v>920</v>
       </c>
       <c r="L18" s="12" t="n">
         <f aca="false">IF(D18=0,0,K18/D18)</f>
-        <v>148.333333333333</v>
+        <v>153.333333333333</v>
       </c>
       <c r="M18" s="9" t="str">
         <f aca="false">IF(Hotels!G18="Booked","Yes",IF(Hotels!G18="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N18" s="31" t="s">
-        <v>105</v>
+        <v>107</v>
+      </c>
+      <c r="O18" s="30" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3096,10 +3160,10 @@
         <v>21</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D19" s="29" t="n">
         <v>4</v>
@@ -3126,19 +3190,22 @@
         <v>80</v>
       </c>
       <c r="K19" s="12" t="n">
-        <f aca="false">G19+H19+I19+J19</f>
-        <v>305</v>
+        <f aca="false">G19+H19+I19+J19+O19</f>
+        <v>325</v>
       </c>
       <c r="L19" s="12" t="n">
         <f aca="false">IF(D19=0,0,K19/D19)</f>
-        <v>76.25</v>
+        <v>81.25</v>
       </c>
       <c r="M19" s="9" t="str">
         <f aca="false">IF(Hotels!G19="Booked","Yes",IF(Hotels!G19="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N19" s="31" t="s">
-        <v>108</v>
+        <v>110</v>
+      </c>
+      <c r="O19" s="30" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3146,7 +3213,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>23</v>
@@ -3176,19 +3243,22 @@
         <v>760</v>
       </c>
       <c r="K20" s="12" t="n">
-        <f aca="false">G20+H20+I20+J20</f>
-        <v>1040</v>
+        <f aca="false">G20+H20+I20+J20+O20</f>
+        <v>1140</v>
       </c>
       <c r="L20" s="12" t="n">
         <f aca="false">IF(D20=0,0,K20/D20)</f>
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="M20" s="9" t="str">
         <f aca="false">IF(Hotels!G20="Booked","Yes",IF(Hotels!G20="Staying with friends","N/A – host","No"))</f>
         <v>N/A – host</v>
       </c>
       <c r="N20" s="31" t="s">
-        <v>110</v>
+        <v>112</v>
+      </c>
+      <c r="O20" s="30" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3196,10 +3266,10 @@
         <v>13</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D21" s="29" t="n">
         <v>8</v>
@@ -3226,19 +3296,22 @@
         <v>384</v>
       </c>
       <c r="K21" s="12" t="n">
-        <f aca="false">G21+H21+I21+J21</f>
-        <v>994</v>
+        <f aca="false">G21+H21+I21+J21+O21</f>
+        <v>1034</v>
       </c>
       <c r="L21" s="12" t="n">
         <f aca="false">IF(D21=0,0,K21/D21)</f>
-        <v>124.25</v>
+        <v>129.25</v>
       </c>
       <c r="M21" s="9" t="str">
         <f aca="false">IF(Hotels!G21="Booked","Yes",IF(Hotels!G21="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N21" s="31" t="s">
-        <v>113</v>
+        <v>115</v>
+      </c>
+      <c r="O21" s="30" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3246,10 +3319,10 @@
         <v>13</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D22" s="29" t="n">
         <v>2</v>
@@ -3276,19 +3349,22 @@
         <v>40</v>
       </c>
       <c r="K22" s="12" t="n">
-        <f aca="false">G22+H22+I22+J22</f>
-        <v>350</v>
+        <f aca="false">G22+H22+I22+J22+O22</f>
+        <v>360</v>
       </c>
       <c r="L22" s="12" t="n">
         <f aca="false">IF(D22=0,0,K22/D22)</f>
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="M22" s="9" t="str">
         <f aca="false">IF(Hotels!G22="Booked","Yes",IF(Hotels!G22="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N22" s="31" t="s">
-        <v>116</v>
+        <v>118</v>
+      </c>
+      <c r="O22" s="30" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3296,10 +3372,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D23" s="29" t="n">
         <v>3</v>
@@ -3326,19 +3402,22 @@
         <v>114</v>
       </c>
       <c r="K23" s="12" t="n">
-        <f aca="false">G23+H23+I23+J23</f>
-        <v>339</v>
+        <f aca="false">G23+H23+I23+J23+O23</f>
+        <v>354</v>
       </c>
       <c r="L23" s="12" t="n">
         <f aca="false">IF(D23=0,0,K23/D23)</f>
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="M23" s="9" t="str">
         <f aca="false">IF(Hotels!G23="Booked","Yes",IF(Hotels!G23="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N23" s="31" t="s">
-        <v>119</v>
+        <v>121</v>
+      </c>
+      <c r="O23" s="30" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3346,10 +3425,10 @@
         <v>13</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D24" s="29" t="n">
         <v>2</v>
@@ -3376,19 +3455,22 @@
         <v>76</v>
       </c>
       <c r="K24" s="12" t="n">
-        <f aca="false">G24+H24+I24+J24</f>
-        <v>396</v>
+        <f aca="false">G24+H24+I24+J24+O24</f>
+        <v>406</v>
       </c>
       <c r="L24" s="12" t="n">
         <f aca="false">IF(D24=0,0,K24/D24)</f>
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="M24" s="9" t="str">
         <f aca="false">IF(Hotels!G24="Booked","Yes",IF(Hotels!G24="Staying with friends","N/A – host","No"))</f>
         <v>No</v>
       </c>
       <c r="N24" s="31" t="s">
-        <v>122</v>
+        <v>124</v>
+      </c>
+      <c r="O24" s="30" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3421,14 +3503,18 @@
       </c>
       <c r="K25" s="16" t="n">
         <f aca="false">SUM(K5:K24)</f>
-        <v>9192.02</v>
+        <v>9647.02</v>
       </c>
       <c r="L25" s="16" t="n">
         <f aca="false">IF(D25=0,0,K25/D25)</f>
-        <v>101.011208791209</v>
+        <v>106.011208791209</v>
       </c>
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
+      <c r="O25" s="16" t="n">
+        <f aca="false">SUM(O5:O24)</f>
+        <v>455</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3467,12 +3553,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3480,43 +3566,43 @@
         <v>4</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D4" s="33" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J4" s="33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K4" s="33" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="L4" s="33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="M4" s="33" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="N4" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3540,10 +3626,10 @@
         <v>46315</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H5" s="39" t="n">
         <v>36</v>
@@ -3553,17 +3639,17 @@
         <v>36</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K5" s="37"/>
       <c r="L5" s="37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3588,10 +3674,10 @@
         <v>46317</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H6" s="39" t="n">
         <v>0</v>
@@ -3601,13 +3687,13 @@
         <v>0</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K6" s="37"/>
       <c r="L6" s="37"/>
       <c r="M6" s="37"/>
       <c r="N6" s="41" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3632,10 +3718,10 @@
         <v>46320</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H7" s="39" t="n">
         <f aca="false">(52.24+239.55)/3</f>
@@ -3646,13 +3732,13 @@
         <v>291.79</v>
       </c>
       <c r="J7" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K7" s="37"/>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
       <c r="N7" s="41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3677,10 +3763,10 @@
         <v>46323</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H8" s="39" t="n">
         <f aca="false">(137.26+66.78)/3</f>
@@ -3691,13 +3777,13 @@
         <v>204.04</v>
       </c>
       <c r="J8" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K8" s="37"/>
       <c r="L8" s="37"/>
       <c r="M8" s="37"/>
       <c r="N8" s="41" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3722,10 +3808,10 @@
         <v>46328</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H9" s="39" t="n">
         <f aca="false">338.05/5</f>
@@ -3736,13 +3822,13 @@
         <v>338.05</v>
       </c>
       <c r="J9" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K9" s="37"/>
       <c r="L9" s="37"/>
       <c r="M9" s="37"/>
       <c r="N9" s="41" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3767,10 +3853,10 @@
         <v>46331</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H10" s="39" t="n">
         <f aca="false">226.17/3</f>
@@ -3781,13 +3867,13 @@
         <v>226.17</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K10" s="37"/>
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
       <c r="N10" s="41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3812,10 +3898,10 @@
         <v>46337</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H11" s="39" t="n">
         <f aca="false">300.97/6</f>
@@ -3826,13 +3912,13 @@
         <v>300.97</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K11" s="37"/>
       <c r="L11" s="37"/>
       <c r="M11" s="37"/>
       <c r="N11" s="41" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3858,7 +3944,7 @@
       </c>
       <c r="F12" s="37"/>
       <c r="G12" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H12" s="39" t="n">
         <v>20</v>
@@ -3872,7 +3958,7 @@
       <c r="L12" s="37"/>
       <c r="M12" s="37"/>
       <c r="N12" s="41" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3898,7 +3984,7 @@
       </c>
       <c r="F13" s="37"/>
       <c r="G13" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H13" s="39" t="n">
         <v>25</v>
@@ -3912,7 +3998,7 @@
       <c r="L13" s="37"/>
       <c r="M13" s="37"/>
       <c r="N13" s="41" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3938,7 +4024,7 @@
       </c>
       <c r="F14" s="37"/>
       <c r="G14" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H14" s="39" t="n">
         <v>45</v>
@@ -3976,7 +4062,7 @@
       </c>
       <c r="F15" s="37"/>
       <c r="G15" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H15" s="39" t="n">
         <v>35</v>
@@ -4014,7 +4100,7 @@
       </c>
       <c r="F16" s="37"/>
       <c r="G16" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H16" s="39" t="n">
         <v>35</v>
@@ -4052,7 +4138,7 @@
       </c>
       <c r="F17" s="37"/>
       <c r="G17" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H17" s="39" t="n">
         <v>25</v>
@@ -4066,7 +4152,7 @@
       <c r="L17" s="37"/>
       <c r="M17" s="37"/>
       <c r="N17" s="41" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4092,7 +4178,7 @@
       </c>
       <c r="F18" s="37"/>
       <c r="G18" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H18" s="39" t="n">
         <v>90</v>
@@ -4106,7 +4192,7 @@
       <c r="L18" s="37"/>
       <c r="M18" s="37"/>
       <c r="N18" s="41" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4132,7 +4218,7 @@
       </c>
       <c r="F19" s="37"/>
       <c r="G19" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H19" s="39" t="n">
         <v>35</v>
@@ -4169,10 +4255,10 @@
         <v>46390</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G20" s="38" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H20" s="39" t="n">
         <v>0</v>
@@ -4182,13 +4268,13 @@
         <v>0</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K20" s="37"/>
       <c r="L20" s="37"/>
       <c r="M20" s="37"/>
       <c r="N20" s="41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4214,7 +4300,7 @@
       </c>
       <c r="F21" s="37"/>
       <c r="G21" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H21" s="39" t="n">
         <v>55</v>
@@ -4228,7 +4314,7 @@
       <c r="L21" s="37"/>
       <c r="M21" s="37"/>
       <c r="N21" s="41" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4254,7 +4340,7 @@
       </c>
       <c r="F22" s="37"/>
       <c r="G22" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H22" s="39" t="n">
         <v>130</v>
@@ -4268,7 +4354,7 @@
       <c r="L22" s="37"/>
       <c r="M22" s="37"/>
       <c r="N22" s="41" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4294,7 +4380,7 @@
       </c>
       <c r="F23" s="37"/>
       <c r="G23" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H23" s="39" t="n">
         <v>55</v>
@@ -4332,7 +4418,7 @@
       </c>
       <c r="F24" s="37"/>
       <c r="G24" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H24" s="39" t="n">
         <v>80</v>
@@ -4346,7 +4432,7 @@
       <c r="L24" s="37"/>
       <c r="M24" s="37"/>
       <c r="N24" s="41" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4379,7 +4465,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C27" s="44" t="str">
         <f aca="false">COUNTIF(G5:G24,"Booked")&amp;" of "&amp;(COUNTA(G5:G24)-COUNTIF(G5:G24,"Staying with friends"))</f>
@@ -4388,7 +4474,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C28" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"Booked",I5:I24)</f>
@@ -4397,7 +4483,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C29" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"To book",I5:I24)+SUMIF(G5:G24,"Shortlisted",I5:I24)</f>
@@ -4452,53 +4538,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="J4" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="K4" s="33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L4" s="33" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M4" s="33" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4509,33 +4595,33 @@
         <v>46313</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F5" s="38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G5" s="38"/>
       <c r="H5" s="38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I5" s="47" t="n">
         <v>667.6</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L5" s="38"/>
       <c r="M5" s="41" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4546,35 +4632,35 @@
         <v>46314</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I6" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K6" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L6" s="38"/>
       <c r="M6" s="41" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4585,35 +4671,35 @@
         <v>46317</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F7" s="38" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H7" s="38" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="I7" s="47" t="n">
         <v>87.7</v>
       </c>
       <c r="J7" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K7" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L7" s="38"/>
       <c r="M7" s="41" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4624,35 +4710,35 @@
         <v>46337</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H8" s="38" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="I8" s="47" t="n">
         <v>211.52</v>
       </c>
       <c r="J8" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K8" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L8" s="38"/>
       <c r="M8" s="41" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4663,29 +4749,29 @@
         <v>46345</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E9" s="38"/>
       <c r="F9" s="38"/>
       <c r="G9" s="38"/>
       <c r="H9" s="38" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I9" s="47" t="n">
         <v>130</v>
       </c>
       <c r="J9" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K9" s="38" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="L9" s="38"/>
       <c r="M9" s="41" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4696,29 +4782,29 @@
         <v>46352</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E10" s="38"/>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
       <c r="H10" s="38" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I10" s="47" t="n">
         <v>130</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L10" s="38"/>
       <c r="M10" s="41" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4729,29 +4815,29 @@
         <v>46360</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="E11" s="38"/>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
       <c r="H11" s="38" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I11" s="47" t="n">
         <v>80</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K11" s="38" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L11" s="38"/>
       <c r="M11" s="41" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4762,29 +4848,29 @@
         <v>46366</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="E12" s="38"/>
       <c r="F12" s="38"/>
       <c r="G12" s="38"/>
       <c r="H12" s="38" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I12" s="47" t="n">
         <v>70</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="L12" s="38"/>
       <c r="M12" s="41" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4795,29 +4881,29 @@
         <v>46370</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E13" s="38"/>
       <c r="F13" s="38"/>
       <c r="G13" s="38"/>
       <c r="H13" s="38" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="I13" s="47" t="n">
         <v>180</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K13" s="38" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="L13" s="38"/>
       <c r="M13" s="41" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4828,29 +4914,29 @@
         <v>46390</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E14" s="38"/>
       <c r="F14" s="38"/>
       <c r="G14" s="38"/>
       <c r="H14" s="38" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="I14" s="47" t="n">
         <v>150</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="L14" s="38"/>
       <c r="M14" s="41" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4861,31 +4947,31 @@
         <v>46405</v>
       </c>
       <c r="C15" s="38" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="G15" s="38" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I15" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K15" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L15" s="38"/>
       <c r="M15" s="41"/>
@@ -4898,35 +4984,35 @@
         <v>46405</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I16" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="L16" s="38"/>
       <c r="M16" s="41" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4951,7 +5037,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I18" s="49" t="n">
         <f aca="false">SUMIF(J5:J16,"Booked",I5:I16)</f>
@@ -4960,7 +5046,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="I19" s="49" t="n">
         <f aca="false">I17-I18</f>
@@ -4969,7 +5055,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -5010,82 +5096,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B5" s="28" t="n">
         <v>281.62</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B6" s="28" t="n">
         <v>62.4</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B7" s="28" t="n">
         <v>13.64</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B8" s="28" t="n">
         <v>100</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5101,225 +5187,225 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C13" s="29"/>
       <c r="D13" s="31"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C14" s="29"/>
       <c r="D14" s="31"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C15" s="29"/>
       <c r="D15" s="31" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C16" s="29"/>
       <c r="D16" s="31" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C17" s="29"/>
       <c r="D17" s="31" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C18" s="29"/>
       <c r="D18" s="31"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C19" s="29"/>
       <c r="D19" s="31" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C20" s="29"/>
       <c r="D20" s="31" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="31" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C22" s="29"/>
       <c r="D22" s="31"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C23" s="29"/>
       <c r="D23" s="31"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C24" s="29"/>
       <c r="D24" s="31" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C25" s="29"/>
       <c r="D25" s="31" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C26" s="29"/>
       <c r="D26" s="31"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C27" s="29"/>
       <c r="D27" s="31"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C28" s="29"/>
       <c r="D28" s="31"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C29" s="29"/>
       <c r="D29" s="31"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C30" s="29"/>
       <c r="D30" s="31"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="31"/>
@@ -5377,17 +5463,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>4</v>
@@ -5396,46 +5482,46 @@
         <v>30</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2788.23</v>
+        <v>2766.01</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C5" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="51" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E5" s="52" t="n">
         <v>667.6</v>
       </c>
       <c r="F5" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I5" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Booked – pay later")</f>
@@ -5444,34 +5530,34 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C6" s="51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D6" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="E6" s="52" t="n">
         <v>281.62</v>
       </c>
       <c r="F6" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2788.23</v>
+        <v>2766.01</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B7" s="51" t="s">
         <v>11</v>
@@ -5480,65 +5566,65 @@
         <v>34</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E7" s="52" t="n">
         <v>36</v>
       </c>
       <c r="F7" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7211.77</v>
+        <v>7233.99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C8" s="51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="E8" s="52" t="n">
         <v>19</v>
       </c>
       <c r="F8" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C9" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D9" s="51" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E9" s="52" t="n">
         <v>87.7</v>
       </c>
       <c r="F9" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B10" s="51" t="s">
         <v>13</v>
@@ -5547,18 +5633,18 @@
         <v>34</v>
       </c>
       <c r="D10" s="51" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="E10" s="52" t="n">
         <v>239.55</v>
       </c>
       <c r="F10" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B11" s="51" t="s">
         <v>13</v>
@@ -5567,38 +5653,38 @@
         <v>34</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E11" s="52" t="n">
         <v>52.24</v>
       </c>
       <c r="F11" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C12" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E12" s="52" t="n">
         <v>211.52</v>
       </c>
       <c r="F12" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B13" s="51" t="s">
         <v>13</v>
@@ -5607,18 +5693,18 @@
         <v>34</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E13" s="52" t="n">
         <v>137.26</v>
       </c>
       <c r="F13" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B14" s="51" t="s">
         <v>13</v>
@@ -5627,18 +5713,18 @@
         <v>34</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E14" s="52" t="n">
         <v>338.05</v>
       </c>
       <c r="F14" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B15" s="51" t="s">
         <v>13</v>
@@ -5647,18 +5733,18 @@
         <v>34</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E15" s="52" t="n">
         <v>66.78</v>
       </c>
       <c r="F15" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="51" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B16" s="51" t="s">
         <v>13</v>
@@ -5667,18 +5753,18 @@
         <v>34</v>
       </c>
       <c r="D16" s="51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="E16" s="52" t="n">
         <v>300.97</v>
       </c>
       <c r="F16" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="51" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B17" s="51" t="s">
         <v>13</v>
@@ -5687,78 +5773,81 @@
         <v>34</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E17" s="52" t="n">
         <v>226.17</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="51" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D18" s="51" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E18" s="52" t="n">
         <v>13.64</v>
       </c>
       <c r="F18" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="E19" s="52" t="n">
         <v>32.4</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B20" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D20" s="51" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="E20" s="52" t="n">
-        <v>3.05</v>
+        <v>2.95</v>
       </c>
       <c r="F20" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>321</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B21" s="51" t="s">
         <v>11</v>
@@ -5767,41 +5856,44 @@
         <v>35</v>
       </c>
       <c r="D21" s="51" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E21" s="52" t="n">
-        <v>14.91</v>
+        <v>3.05</v>
       </c>
       <c r="F21" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>323</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B22" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C22" s="51" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D22" s="51" t="s">
-        <v>320</v>
+        <v>35</v>
       </c>
       <c r="E22" s="52" t="n">
-        <v>2.95</v>
+        <v>14.91</v>
       </c>
       <c r="F22" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="51" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="B23" s="51" t="s">
         <v>11</v>
@@ -5810,21 +5902,21 @@
         <v>35</v>
       </c>
       <c r="D23" s="51" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="E23" s="52" t="n">
-        <v>3.05</v>
+        <v>3.4</v>
       </c>
       <c r="F23" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="51" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="B24" s="51" t="s">
         <v>11</v>
@@ -5833,44 +5925,44 @@
         <v>35</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>35</v>
+        <v>328</v>
       </c>
       <c r="E24" s="52" t="n">
-        <v>14.91</v>
+        <v>2.55</v>
       </c>
       <c r="F24" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="51" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B25" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C25" s="51" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="E25" s="52" t="n">
-        <v>3.4</v>
+        <v>5.9</v>
       </c>
       <c r="F25" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="51" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B26" s="51" t="s">
         <v>11</v>
@@ -5879,67 +5971,67 @@
         <v>35</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="E26" s="52" t="n">
-        <v>2.55</v>
+        <v>8.5</v>
       </c>
       <c r="F26" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="51" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B27" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C27" s="51" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>320</v>
+        <v>333</v>
       </c>
       <c r="E27" s="52" t="n">
-        <v>5.9</v>
+        <v>8.87</v>
       </c>
       <c r="F27" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="51" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B28" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="51" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E28" s="52" t="n">
-        <v>8.5</v>
+        <v>3.4</v>
       </c>
       <c r="F28" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="51" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B29" s="51" t="s">
         <v>11</v>
@@ -5948,86 +6040,41 @@
         <v>35</v>
       </c>
       <c r="D29" s="51" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="E29" s="52" t="n">
-        <v>8.87</v>
+        <v>1.98</v>
       </c>
       <c r="F29" s="51" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="B30" s="51" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="51" t="s">
-        <v>37</v>
-      </c>
-      <c r="D30" s="51" t="s">
-        <v>334</v>
-      </c>
-      <c r="E30" s="52" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="F30" s="51" t="s">
-        <v>41</v>
-      </c>
-      <c r="J30" s="1" t="s">
-        <v>335</v>
-      </c>
+      <c r="A30" s="51"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="51"/>
+      <c r="D30" s="51"/>
+      <c r="E30" s="52"/>
+      <c r="F30" s="51"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="51" t="s">
-        <v>324</v>
-      </c>
-      <c r="B31" s="51" t="s">
-        <v>11</v>
-      </c>
-      <c r="C31" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="D31" s="51" t="s">
-        <v>336</v>
-      </c>
-      <c r="E31" s="52" t="n">
-        <v>1.98</v>
-      </c>
-      <c r="F31" s="51" t="s">
-        <v>41</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>337</v>
-      </c>
+      <c r="A31" s="51"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="51"/>
+      <c r="D31" s="51"/>
+      <c r="E31" s="52"/>
+      <c r="F31" s="51"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="51" t="s">
-        <v>338</v>
-      </c>
-      <c r="B32" s="51" t="s">
-        <v>11</v>
-      </c>
-      <c r="C32" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="D32" s="51" t="s">
-        <v>339</v>
-      </c>
-      <c r="E32" s="52" t="n">
-        <v>4.26</v>
-      </c>
-      <c r="F32" s="51" t="s">
-        <v>41</v>
-      </c>
-      <c r="J32" s="1" t="s">
-        <v>340</v>
-      </c>
+      <c r="A32" s="51"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="52"/>
+      <c r="F32" s="51"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="51"/>
@@ -13757,22 +13804,8 @@
       <c r="E998" s="52"/>
       <c r="F998" s="51"/>
     </row>
-    <row r="999" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A999" s="51"/>
-      <c r="B999" s="51"/>
-      <c r="C999" s="51"/>
-      <c r="D999" s="51"/>
-      <c r="E999" s="52"/>
-      <c r="F999" s="51"/>
-    </row>
-    <row r="1000" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1000" s="51"/>
-      <c r="B1000" s="51"/>
-      <c r="C1000" s="51"/>
-      <c r="D1000" s="51"/>
-      <c r="E1000" s="52"/>
-      <c r="F1000" s="51"/>
-    </row>
+    <row r="999" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="1000" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B5:B1000" type="list">
@@ -13780,7 +13813,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C1000" type="list">
-      <formula1>"Flights,Accommodation,Food,Local transport,Activities,Insurance &amp; admin,Other"</formula1>
+      <formula1>"Flights,Accommodation,Food,Local transport,Activities,Shopping &amp; misc,Insurance &amp; admin,Other"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F1000" type="list">

</xml_diff>

<commit_message>
Sync Tracker with spend log (2 added, 0 updated, 0 removed)
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="345">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -1042,6 +1042,24 @@
   </si>
   <si>
     <t xml:space="preserve">mvgm1pq2sx7l</t>
+  </si>
+  <si>
+    <t xml:space="preserve">21/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvha28vt2umu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22/10/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Narita Express</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mvhbcrzpy1g5</t>
   </si>
 </sst>
 </file>
@@ -1797,11 +1815,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>91.51</v>
+        <v>95.77</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">D7+D13-F7</f>
-        <v>1244.49</v>
+        <v>1240.23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1825,11 +1843,11 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>1361.02</v>
+        <v>1384.27</v>
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">D8+D14-F8</f>
-        <v>3659</v>
+        <v>3635.75</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2091,11 +2109,11 @@
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
-        <v>43.26</v>
+        <v>47.52</v>
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3346.74</v>
+        <v>3342.48</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
@@ -2112,11 +2130,11 @@
       </c>
       <c r="C23" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A23)</f>
-        <v>8.85</v>
+        <v>32.1</v>
       </c>
       <c r="D23" s="18" t="n">
         <f aca="false">B23-C23</f>
-        <v>961.15</v>
+        <v>937.9</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B23/$B$3)</f>
@@ -2217,11 +2235,11 @@
       </c>
       <c r="C28" s="24" t="n">
         <f aca="false">SUM(C20:C27)</f>
-        <v>2766.01</v>
+        <v>2793.52</v>
       </c>
       <c r="D28" s="24" t="n">
         <f aca="false">SUM(D20:D27)</f>
-        <v>7233.99</v>
+        <v>7206.48</v>
       </c>
       <c r="E28" s="25" t="n">
         <f aca="false">SUM(E20:E27)</f>
@@ -2246,7 +2264,7 @@
       </c>
       <c r="B32" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2766.01</v>
+        <v>2793.52</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2264,7 +2282,7 @@
       </c>
       <c r="B34" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7233.99</v>
+        <v>7206.48</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2293,7 +2311,7 @@
       </c>
       <c r="B40" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2766.01</v>
+        <v>2793.52</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2302,7 +2320,7 @@
       </c>
       <c r="B41" s="27" t="n">
         <f aca="false">B39-B40</f>
-        <v>5268.26</v>
+        <v>5240.75</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5495,7 +5513,7 @@
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2766.01</v>
+        <v>2793.52</v>
       </c>
       <c r="J4" s="7" t="s">
         <v>293</v>
@@ -5552,7 +5570,7 @@
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2766.01</v>
+        <v>2793.52</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5579,7 +5597,7 @@
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7233.99</v>
+        <v>7206.48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6053,20 +6071,50 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="51"/>
-      <c r="B30" s="51"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="51"/>
-      <c r="E30" s="52"/>
-      <c r="F30" s="51"/>
+      <c r="A30" s="51" t="s">
+        <v>339</v>
+      </c>
+      <c r="B30" s="51" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="51" t="s">
+        <v>35</v>
+      </c>
+      <c r="D30" s="51" t="s">
+        <v>340</v>
+      </c>
+      <c r="E30" s="52" t="n">
+        <v>4.26</v>
+      </c>
+      <c r="F30" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="J30" s="1" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="51"/>
-      <c r="B31" s="51"/>
-      <c r="C31" s="51"/>
-      <c r="D31" s="51"/>
-      <c r="E31" s="52"/>
-      <c r="F31" s="51"/>
+      <c r="A31" s="51" t="s">
+        <v>342</v>
+      </c>
+      <c r="B31" s="51" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="51" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="51" t="s">
+        <v>343</v>
+      </c>
+      <c r="E31" s="52" t="n">
+        <v>23.25</v>
+      </c>
+      <c r="F31" s="51" t="s">
+        <v>42</v>
+      </c>
+      <c r="J31" s="1" t="s">
+        <v>344</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="51"/>

</xml_diff>

<commit_message>
Itinerary: Kuala Lumpur 4 nights (26–30 Nov), Johor 4 nights (30 Nov–4 Dec)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018LrmqD6uz8F6WnijcfuM7x
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -327,7 +327,7 @@
     <t xml:space="preserve">Kuala Lumpur</t>
   </si>
   <si>
-    <t xml:space="preserve">26 – 29 Nov</t>
+    <t xml:space="preserve">26 – 30 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">See friend 27 Nov</t>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">Johor + Singapore day trips</t>
   </si>
   <si>
-    <t xml:space="preserve">29 Nov – 4 Dec</t>
+    <t xml:space="preserve">30 Nov – 4 Dec</t>
   </si>
   <si>
     <t xml:space="preserve">Food incl. £90 Singapore treat. SG Arrival Card each crossing</t>
@@ -831,7 +831,7 @@
     <t xml:space="preserve">Proof of leaving Taiwan</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm Johor friend dates (29 Nov–4 Dec)</t>
+    <t xml:space="preserve">Confirm Johor friend dates (30 Nov–4 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Soon</t>
@@ -1066,13 +1066,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\£#,##0;&quot;(£&quot;#,##0\);\-"/>
-    <numFmt numFmtId="166" formatCode="General"/>
-    <numFmt numFmtId="167" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="ddd\ d\ mmm\ yyyy"/>
+    <numFmt numFmtId="166" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="ddd\ d\ mmm\ yyyy"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -1299,7 +1298,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1331,7 +1330,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1339,15 +1342,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1355,7 +1358,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1363,19 +1366,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1403,11 +1402,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1451,19 +1450,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1471,7 +1470,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1564,34 +1563,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1737,7 +1736,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G43"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
@@ -1919,11 +1918,11 @@
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">SUM(Itinerary!K16:K17)</f>
-        <v>736</v>
+        <v>728</v>
       </c>
       <c r="E11" s="11" t="n">
         <f aca="false">IF(C11=0,0,D11/C11)</f>
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1931,7 +1930,7 @@
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">D11-F11</f>
-        <v>736</v>
+        <v>728</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1970,11 +1969,11 @@
         <v>23</v>
       </c>
       <c r="C13" s="9" t="n">
-        <f aca="false">SUM(Itinerary!D20:D20)</f>
+        <f aca="false">SUM(Itinerary!D20)</f>
         <v>20</v>
       </c>
       <c r="D13" s="10" t="n">
-        <f aca="false">SUM(Itinerary!K20:K20)</f>
+        <f aca="false">SUM(Itinerary!K20)</f>
         <v>1140</v>
       </c>
       <c r="E13" s="11" t="n">
@@ -2021,11 +2020,11 @@
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">SUM(D7:D14)</f>
-        <v>9647.02</v>
+        <v>9639.02</v>
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">IF(C15=0,0,D15/C15)</f>
-        <v>106.011208791209</v>
+        <v>105.923296703297</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="15"/>
@@ -2084,7 +2083,7 @@
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">Itinerary!I25</f>
-        <v>3802.02</v>
+        <v>3812.02</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A21)</f>
@@ -2092,11 +2091,11 @@
       </c>
       <c r="D21" s="18" t="n">
         <f aca="false">B21-C21</f>
-        <v>2405</v>
+        <v>2415</v>
       </c>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B21/$B$3)</f>
-        <v>0.380202</v>
+        <v>0.381202</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2105,7 +2104,7 @@
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">Itinerary!J25</f>
-        <v>3390</v>
+        <v>3372</v>
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
@@ -2113,11 +2112,11 @@
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3342.48</v>
+        <v>3324.48</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
-        <v>0.339</v>
+        <v>0.3372</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2210,7 +2209,7 @@
       </c>
       <c r="B27" s="21" t="n">
         <f aca="false">$B$3-SUM(B20:B26)</f>
-        <v>-1811.5</v>
+        <v>-1803.5</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,"Other")</f>
@@ -2218,11 +2217,11 @@
       </c>
       <c r="D27" s="22" t="n">
         <f aca="false">B27-C27</f>
-        <v>-1811.5</v>
+        <v>-1803.5</v>
       </c>
       <c r="E27" s="23" t="n">
         <f aca="false">IF($B$3=0,0,B27/$B$3)</f>
-        <v>-0.18115</v>
+        <v>-0.18035</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2249,7 +2248,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="str">
         <f aca="false">IF(B27&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B27,"£#,##0"),IF(B27&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
-        <v>⚠ Plan is over budget by £1,812</v>
+        <v>⚠ Plan is over budget by £1,804</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2338,7 +2337,7 @@
       </c>
       <c r="B43" s="27" t="n">
         <f aca="false">MAX(0,SUM(B20:B26)-B39)</f>
-        <v>3777.23</v>
+        <v>3769.23</v>
       </c>
     </row>
   </sheetData>
@@ -2358,7 +2357,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O25"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
@@ -3025,7 +3024,7 @@
         <v>100</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" s="10" t="n">
         <f aca="false">Hotels!H16</f>
@@ -3042,19 +3041,19 @@
       </c>
       <c r="I16" s="12" t="n">
         <f aca="false">D16*E16</f>
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="J16" s="12" t="n">
         <f aca="false">D16*F16</f>
-        <v>66</v>
+        <v>88</v>
       </c>
       <c r="K16" s="12" t="n">
         <f aca="false">G16+H16+I16+J16+O16</f>
-        <v>246</v>
+        <v>308</v>
       </c>
       <c r="L16" s="12" t="n">
         <f aca="false">IF(D16=0,0,K16/D16)</f>
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="M16" s="9" t="str">
         <f aca="false">IF(Hotels!G16="Booked","Yes",IF(Hotels!G16="Staying with friends","N/A – host","No"))</f>
@@ -3064,7 +3063,7 @@
         <v>101</v>
       </c>
       <c r="O16" s="30" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3078,7 +3077,7 @@
         <v>103</v>
       </c>
       <c r="D17" s="29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">Hotels!H17</f>
@@ -3095,19 +3094,19 @@
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">D17*E17</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">D17*F17</f>
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">G17+H17+I17+J17+O17</f>
-        <v>490</v>
+        <v>420</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">IF(D17=0,0,K17/D17)</f>
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="M17" s="9" t="str">
         <f aca="false">IF(Hotels!G17="Booked","Yes",IF(Hotels!G17="Staying with friends","N/A – host","No"))</f>
@@ -3117,7 +3116,7 @@
         <v>104</v>
       </c>
       <c r="O17" s="30" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3513,19 +3512,19 @@
       </c>
       <c r="I25" s="16" t="n">
         <f aca="false">SUM(I5:I24)</f>
-        <v>3802.02</v>
+        <v>3812.02</v>
       </c>
       <c r="J25" s="16" t="n">
         <f aca="false">SUM(J5:J24)</f>
-        <v>3390</v>
+        <v>3372</v>
       </c>
       <c r="K25" s="16" t="n">
         <f aca="false">SUM(K5:K24)</f>
-        <v>9647.02</v>
+        <v>9639.02</v>
       </c>
       <c r="L25" s="16" t="n">
         <f aca="false">IF(D25=0,0,K25/D25)</f>
-        <v>106.011208791209</v>
+        <v>105.923296703297</v>
       </c>
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
@@ -3551,7 +3550,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N29"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
@@ -4110,11 +4109,11 @@
       </c>
       <c r="D16" s="34" t="n">
         <f aca="false">Itinerary!D16</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E16" s="36" t="n">
         <f aca="false">C16+D16</f>
-        <v>46355</v>
+        <v>46356</v>
       </c>
       <c r="F16" s="37"/>
       <c r="G16" s="38" t="s">
@@ -4125,7 +4124,7 @@
       </c>
       <c r="I16" s="40" t="n">
         <f aca="false">D16*H16</f>
-        <v>105</v>
+        <v>140</v>
       </c>
       <c r="J16" s="38"/>
       <c r="K16" s="37"/>
@@ -4144,11 +4143,11 @@
       </c>
       <c r="C17" s="36" t="n">
         <f aca="false">E16</f>
-        <v>46355</v>
+        <v>46356</v>
       </c>
       <c r="D17" s="34" t="n">
         <f aca="false">Itinerary!D17</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E17" s="36" t="n">
         <f aca="false">C17+D17</f>
@@ -4163,7 +4162,7 @@
       </c>
       <c r="I17" s="40" t="n">
         <f aca="false">D17*H17</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J17" s="38"/>
       <c r="K17" s="37"/>
@@ -4469,7 +4468,7 @@
       <c r="H25" s="42"/>
       <c r="I25" s="43" t="n">
         <f aca="false">SUM(I5:I24)</f>
-        <v>3802.02</v>
+        <v>3812.02</v>
       </c>
       <c r="J25" s="42"/>
       <c r="K25" s="42"/>
@@ -4505,7 +4504,7 @@
       </c>
       <c r="C29" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"To book",I5:I24)+SUMIF(G5:G24,"Shortlisted",I5:I24)</f>
-        <v>2405</v>
+        <v>2415</v>
       </c>
     </row>
   </sheetData>
@@ -4540,7 +4539,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17"/>
@@ -5104,7 +5103,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
@@ -5465,7 +5464,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>

</xml_diff>

<commit_message>
Itinerary: Hanoi 4, Taipei 5, Johor 30 Nov–5 Dec, Thailand beach 5–10 Dec
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018LrmqD6uz8F6WnijcfuM7x
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -75,25 +75,25 @@
     <t xml:space="preserve">Vietnam</t>
   </si>
   <si>
-    <t xml:space="preserve">11 – 19 Nov</t>
+    <t xml:space="preserve">11 – 18 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">Taiwan</t>
   </si>
   <si>
-    <t xml:space="preserve">19 – 26 Nov</t>
+    <t xml:space="preserve">18 – 26 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">Malaysia &amp; Singapore</t>
   </si>
   <si>
-    <t xml:space="preserve">26 Nov – 4 Dec</t>
+    <t xml:space="preserve">26 Nov – 5 Dec</t>
   </si>
   <si>
     <t xml:space="preserve">Thailand</t>
   </si>
   <si>
-    <t xml:space="preserve">4 – 14 Dec</t>
+    <t xml:space="preserve">5 – 14 Dec</t>
   </si>
   <si>
     <t xml:space="preserve">14 Dec – 3 Jan</t>
@@ -300,7 +300,7 @@
     <t xml:space="preserve">Hanoi</t>
   </si>
   <si>
-    <t xml:space="preserve">14 – 19 Nov</t>
+    <t xml:space="preserve">14 – 18 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">Food incl. £45 tasting-menu treat. Optional Ha Long Bay day trip (~£50). ~45 min to airport</t>
@@ -309,7 +309,7 @@
     <t xml:space="preserve">Taipei</t>
   </si>
   <si>
-    <t xml:space="preserve">19 – 23 Nov</t>
+    <t xml:space="preserve">18 – 23 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">Food incl. £90 tasting-menu treat. Jiufen, Beitou hot springs</t>
@@ -336,7 +336,7 @@
     <t xml:space="preserve">Johor + Singapore day trips</t>
   </si>
   <si>
-    <t xml:space="preserve">30 Nov – 4 Dec</t>
+    <t xml:space="preserve">30 Nov – 5 Dec</t>
   </si>
   <si>
     <t xml:space="preserve">Food incl. £90 Singapore treat. SG Arrival Card each crossing</t>
@@ -345,7 +345,7 @@
     <t xml:space="preserve">Beach resort – Andaman coast</t>
   </si>
   <si>
-    <t xml:space="preserve">4 – 10 Dec</t>
+    <t xml:space="preserve">5 – 10 Dec</t>
   </si>
   <si>
     <t xml:space="preserve">Peak dry season. Food incl. £60 seafood treat. Khao Lak / Phuket / Krabi</t>
@@ -822,7 +822,7 @@
     <t xml:space="preserve">Book Tam Coc resort + airport pickup, and Hanoi hotel</t>
   </si>
   <si>
-    <t xml:space="preserve">Book Hanoi → Taipei (19 Nov)</t>
+    <t xml:space="preserve">Book Hanoi → Taipei (18 Nov)</t>
   </si>
   <si>
     <t xml:space="preserve">Book Kaohsiung → KL (26 Nov)</t>
@@ -831,7 +831,7 @@
     <t xml:space="preserve">Proof of leaving Taiwan</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm Johor friend dates (30 Nov–4 Dec)</t>
+    <t xml:space="preserve">Confirm Johor friend dates (30 Nov–5 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Soon</t>
@@ -846,7 +846,7 @@
     <t xml:space="preserve">Book KL + Johor stays</t>
   </si>
   <si>
-    <t xml:space="preserve">Choose Thailand resort (4–10 Dec) + Chiang Mai (10–14 Dec)</t>
+    <t xml:space="preserve">Choose Thailand resort (5–10 Dec) + Chiang Mai (10–14 Dec)</t>
   </si>
   <si>
     <t xml:space="preserve">Peak season – book ahead</t>
@@ -876,7 +876,7 @@
     <t xml:space="preserve">Taiwan online arrival card</t>
   </si>
   <si>
-    <t xml:space="preserve">Before 19 Nov</t>
+    <t xml:space="preserve">Before 18 Nov</t>
   </si>
   <si>
     <t xml:space="preserve">Malaysia Digital Arrival Card (MDAC)</t>
@@ -1858,15 +1858,15 @@
       </c>
       <c r="C9" s="9" t="n">
         <f aca="false">SUM(Itinerary!D12:D13)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">SUM(Itinerary!K12:K13)</f>
-        <v>575</v>
+        <v>518</v>
       </c>
       <c r="E9" s="11" t="n">
         <f aca="false">IF(C9=0,0,D9/C9)</f>
-        <v>71.875</v>
+        <v>74</v>
       </c>
       <c r="F9" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Vietnam",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="G9" s="12" t="n">
         <f aca="false">D9-F9</f>
-        <v>575</v>
+        <v>518</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1886,15 +1886,15 @@
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">SUM(Itinerary!D14:D15)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">SUM(Itinerary!K14:K15)</f>
-        <v>735</v>
+        <v>832.5</v>
       </c>
       <c r="E10" s="11" t="n">
         <f aca="false">IF(C10=0,0,D10/C10)</f>
-        <v>105</v>
+        <v>104.0625</v>
       </c>
       <c r="F10" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Taiwan",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G10" s="12" t="n">
         <f aca="false">D10-F10</f>
-        <v>735</v>
+        <v>832.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1914,15 +1914,15 @@
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">SUM(Itinerary!D16:D17)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">SUM(Itinerary!K16:K17)</f>
-        <v>728</v>
+        <v>798</v>
       </c>
       <c r="E11" s="11" t="n">
         <f aca="false">IF(C11=0,0,D11/C11)</f>
-        <v>91</v>
+        <v>88.6666666666667</v>
       </c>
       <c r="F11" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Malaysia &amp; Singapore",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="G11" s="12" t="n">
         <f aca="false">D11-F11</f>
-        <v>728</v>
+        <v>798</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1942,15 +1942,15 @@
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">SUM(Itinerary!D18:D19)</f>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D12" s="10" t="n">
         <f aca="false">SUM(Itinerary!K18:K19)</f>
-        <v>1245</v>
+        <v>1105</v>
       </c>
       <c r="E12" s="11" t="n">
         <f aca="false">IF(C12=0,0,D12/C12)</f>
-        <v>124.5</v>
+        <v>122.777777777778</v>
       </c>
       <c r="F12" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Thailand",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="G12" s="12" t="n">
         <f aca="false">D12-F12</f>
-        <v>1245</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2020,11 +2020,11 @@
       </c>
       <c r="D15" s="16" t="n">
         <f aca="false">SUM(D7:D14)</f>
-        <v>9639.02</v>
+        <v>9609.52</v>
       </c>
       <c r="E15" s="16" t="n">
         <f aca="false">IF(C15=0,0,D15/C15)</f>
-        <v>105.923296703297</v>
+        <v>105.599120879121</v>
       </c>
       <c r="F15" s="15"/>
       <c r="G15" s="15"/>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="B21" s="17" t="n">
         <f aca="false">Itinerary!I25</f>
-        <v>3812.02</v>
+        <v>3767.02</v>
       </c>
       <c r="C21" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A21)</f>
@@ -2091,11 +2091,11 @@
       </c>
       <c r="D21" s="18" t="n">
         <f aca="false">B21-C21</f>
-        <v>2415</v>
+        <v>2370</v>
       </c>
       <c r="E21" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B21/$B$3)</f>
-        <v>0.381202</v>
+        <v>0.376702</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2104,7 +2104,7 @@
       </c>
       <c r="B22" s="17" t="n">
         <f aca="false">Itinerary!J25</f>
-        <v>3372</v>
+        <v>3387.5</v>
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
@@ -2112,11 +2112,11 @@
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3324.48</v>
+        <v>3339.98</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
-        <v>0.3372</v>
+        <v>0.33875</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="B27" s="21" t="n">
         <f aca="false">$B$3-SUM(B20:B26)</f>
-        <v>-1803.5</v>
+        <v>-1774</v>
       </c>
       <c r="C27" s="22" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,"Other")</f>
@@ -2217,11 +2217,11 @@
       </c>
       <c r="D27" s="22" t="n">
         <f aca="false">B27-C27</f>
-        <v>-1803.5</v>
+        <v>-1774</v>
       </c>
       <c r="E27" s="23" t="n">
         <f aca="false">IF($B$3=0,0,B27/$B$3)</f>
-        <v>-0.18035</v>
+        <v>-0.1774</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2248,7 +2248,7 @@
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="str">
         <f aca="false">IF(B27&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B27,"£#,##0"),IF(B27&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
-        <v>⚠ Plan is over budget by £1,804</v>
+        <v>⚠ Plan is over budget by £1,774</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2337,7 +2337,7 @@
       </c>
       <c r="B43" s="27" t="n">
         <f aca="false">MAX(0,SUM(B20:B26)-B39)</f>
-        <v>3769.23</v>
+        <v>3739.73</v>
       </c>
     </row>
   </sheetData>
@@ -2865,7 +2865,7 @@
         <v>91</v>
       </c>
       <c r="D13" s="29" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="10" t="n">
         <f aca="false">Hotels!H13</f>
@@ -2882,19 +2882,19 @@
       </c>
       <c r="I13" s="12" t="n">
         <f aca="false">D13*E13</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J13" s="12" t="n">
         <f aca="false">D13*F13</f>
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="K13" s="12" t="n">
         <f aca="false">G13+H13+I13+J13+O13</f>
-        <v>370</v>
+        <v>313</v>
       </c>
       <c r="L13" s="12" t="n">
         <f aca="false">IF(D13=0,0,K13/D13)</f>
-        <v>74</v>
+        <v>78.25</v>
       </c>
       <c r="M13" s="9" t="str">
         <f aca="false">IF(Hotels!G13="Booked","Yes",IF(Hotels!G13="Staying with friends","N/A – host","No"))</f>
@@ -2904,7 +2904,7 @@
         <v>92</v>
       </c>
       <c r="O13" s="30" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2918,7 +2918,7 @@
         <v>94</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="10" t="n">
         <f aca="false">Hotels!H14</f>
@@ -2935,19 +2935,19 @@
       </c>
       <c r="I14" s="12" t="n">
         <f aca="false">D14*E14</f>
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="J14" s="12" t="n">
         <f aca="false">D14*F14</f>
-        <v>190</v>
+        <v>237.5</v>
       </c>
       <c r="K14" s="12" t="n">
         <f aca="false">G14+H14+I14+J14+O14</f>
-        <v>460</v>
+        <v>557.5</v>
       </c>
       <c r="L14" s="12" t="n">
         <f aca="false">IF(D14=0,0,K14/D14)</f>
-        <v>115</v>
+        <v>111.5</v>
       </c>
       <c r="M14" s="9" t="str">
         <f aca="false">IF(Hotels!G14="Booked","Yes",IF(Hotels!G14="Staying with friends","N/A – host","No"))</f>
@@ -2957,7 +2957,7 @@
         <v>95</v>
       </c>
       <c r="O14" s="30" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3077,7 +3077,7 @@
         <v>103</v>
       </c>
       <c r="D17" s="29" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">Hotels!H17</f>
@@ -3094,19 +3094,19 @@
       </c>
       <c r="I17" s="12" t="n">
         <f aca="false">D17*E17</f>
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="J17" s="12" t="n">
         <f aca="false">D17*F17</f>
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">G17+H17+I17+J17+O17</f>
-        <v>420</v>
+        <v>490</v>
       </c>
       <c r="L17" s="12" t="n">
         <f aca="false">IF(D17=0,0,K17/D17)</f>
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="M17" s="9" t="str">
         <f aca="false">IF(Hotels!G17="Booked","Yes",IF(Hotels!G17="Staying with friends","N/A – host","No"))</f>
@@ -3116,7 +3116,7 @@
         <v>104</v>
       </c>
       <c r="O17" s="30" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3130,7 +3130,7 @@
         <v>106</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="10" t="n">
         <f aca="false">Hotels!H18</f>
@@ -3147,19 +3147,19 @@
       </c>
       <c r="I18" s="12" t="n">
         <f aca="false">D18*E18</f>
-        <v>540</v>
+        <v>450</v>
       </c>
       <c r="J18" s="12" t="n">
         <f aca="false">D18*F18</f>
-        <v>270</v>
+        <v>225</v>
       </c>
       <c r="K18" s="12" t="n">
         <f aca="false">G18+H18+I18+J18+O18</f>
-        <v>920</v>
+        <v>780</v>
       </c>
       <c r="L18" s="12" t="n">
         <f aca="false">IF(D18=0,0,K18/D18)</f>
-        <v>153.333333333333</v>
+        <v>156</v>
       </c>
       <c r="M18" s="9" t="str">
         <f aca="false">IF(Hotels!G18="Booked","Yes",IF(Hotels!G18="Staying with friends","N/A – host","No"))</f>
@@ -3169,7 +3169,7 @@
         <v>107</v>
       </c>
       <c r="O18" s="30" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3512,19 +3512,19 @@
       </c>
       <c r="I25" s="16" t="n">
         <f aca="false">SUM(I5:I24)</f>
-        <v>3812.02</v>
+        <v>3767.02</v>
       </c>
       <c r="J25" s="16" t="n">
         <f aca="false">SUM(J5:J24)</f>
-        <v>3372</v>
+        <v>3387.5</v>
       </c>
       <c r="K25" s="16" t="n">
         <f aca="false">SUM(K5:K24)</f>
-        <v>9639.02</v>
+        <v>9609.52</v>
       </c>
       <c r="L25" s="16" t="n">
         <f aca="false">IF(D25=0,0,K25/D25)</f>
-        <v>105.923296703297</v>
+        <v>105.599120879121</v>
       </c>
       <c r="M25" s="15"/>
       <c r="N25" s="15"/>
@@ -3993,11 +3993,11 @@
       </c>
       <c r="D13" s="34" t="n">
         <f aca="false">Itinerary!D13</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="36" t="n">
         <f aca="false">C13+D13</f>
-        <v>46345</v>
+        <v>46344</v>
       </c>
       <c r="F13" s="37"/>
       <c r="G13" s="38" t="s">
@@ -4008,7 +4008,7 @@
       </c>
       <c r="I13" s="40" t="n">
         <f aca="false">D13*H13</f>
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J13" s="38"/>
       <c r="K13" s="37"/>
@@ -4029,11 +4029,11 @@
       </c>
       <c r="C14" s="36" t="n">
         <f aca="false">E13</f>
-        <v>46345</v>
+        <v>46344</v>
       </c>
       <c r="D14" s="34" t="n">
         <f aca="false">Itinerary!D14</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="36" t="n">
         <f aca="false">C14+D14</f>
@@ -4048,7 +4048,7 @@
       </c>
       <c r="I14" s="40" t="n">
         <f aca="false">D14*H14</f>
-        <v>180</v>
+        <v>225</v>
       </c>
       <c r="J14" s="38"/>
       <c r="K14" s="37"/>
@@ -4147,11 +4147,11 @@
       </c>
       <c r="D17" s="34" t="n">
         <f aca="false">Itinerary!D17</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E17" s="36" t="n">
         <f aca="false">C17+D17</f>
-        <v>46360</v>
+        <v>46361</v>
       </c>
       <c r="F17" s="37"/>
       <c r="G17" s="38" t="s">
@@ -4162,7 +4162,7 @@
       </c>
       <c r="I17" s="40" t="n">
         <f aca="false">D17*H17</f>
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="J17" s="38"/>
       <c r="K17" s="37"/>
@@ -4183,11 +4183,11 @@
       </c>
       <c r="C18" s="36" t="n">
         <f aca="false">E17</f>
-        <v>46360</v>
+        <v>46361</v>
       </c>
       <c r="D18" s="34" t="n">
         <f aca="false">Itinerary!D18</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E18" s="36" t="n">
         <f aca="false">C18+D18</f>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="I18" s="40" t="n">
         <f aca="false">D18*H18</f>
-        <v>540</v>
+        <v>450</v>
       </c>
       <c r="J18" s="38"/>
       <c r="K18" s="37"/>
@@ -4468,7 +4468,7 @@
       <c r="H25" s="42"/>
       <c r="I25" s="43" t="n">
         <f aca="false">SUM(I5:I24)</f>
-        <v>3812.02</v>
+        <v>3767.02</v>
       </c>
       <c r="J25" s="42"/>
       <c r="K25" s="42"/>
@@ -4504,7 +4504,7 @@
       </c>
       <c r="C29" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"To book",I5:I24)+SUMIF(G5:G24,"Shortlisted",I5:I24)</f>
-        <v>2415</v>
+        <v>2370</v>
       </c>
     </row>
   </sheetData>
@@ -4763,7 +4763,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="35" t="n">
-        <v>46345</v>
+        <v>46344</v>
       </c>
       <c r="C9" s="38" t="s">
         <v>204</v>
@@ -4829,7 +4829,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="35" t="n">
-        <v>46360</v>
+        <v>46361</v>
       </c>
       <c r="C11" s="38" t="s">
         <v>213</v>

</xml_diff>

<commit_message>
Budget accuracy + new Daily cards
- Duplicates: hand-typed Tracker rows matching a logged spend are counted once and merged on sync; repeats warned when logging and flagged in the day list
- Days with nothing logged count at plan until confirmed (Nothing spent)
- Trains & intercity budget line (Itinerary column P, £231 moved from Local transport) and 🚄 log type; Narita Express re-tagged
- To book & do card, cash wallet, end-of-stay wrap-up
- push.sh: commit + push without spreadsheet merge errors; workflow also re-syncs when the spreadsheet is pushed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018LrmqD6uz8F6WnijcfuM7x
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="583" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="352">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Ground costs only (accommodation, food, local transport, activities, shopping &amp; misc). Korea &amp; Japan appear twice – spend is combined on their first row.</t>
+    <t xml:space="preserve">Ground costs only (accommodation, food, local transport, trains &amp; intercity, activities, shopping &amp; misc). Korea &amp; Japan appear twice – spend is combined on their first row.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Budget by category</t>
@@ -138,6 +138,9 @@
     <t xml:space="preserve">Local transport</t>
   </si>
   <si>
+    <t xml:space="preserve">Trains &amp; intercity</t>
+  </si>
+  <si>
     <t xml:space="preserve">Activities</t>
   </si>
   <si>
@@ -225,6 +228,9 @@
     <t xml:space="preserve">Shopping &amp; misc (£)</t>
   </si>
   <si>
+    <t xml:space="preserve">Trains &amp; intercity (£)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Incheon – Incheon Airport Hotel Seattle</t>
   </si>
   <si>
@@ -249,7 +255,7 @@
     <t xml:space="preserve">22 – 25 Oct</t>
   </si>
   <si>
-    <t xml:space="preserve">MARATHON 25 Oct. Arrive Narita 15:30 on 22 Oct – Narita Express / limousine bus (~90 min)</t>
+    <t xml:space="preserve">MARATHON 25 Oct. Arrive Narita 15:30 on 22 Oct. Trains: Narita Express to Yokohama (~£23).</t>
   </si>
   <si>
     <t xml:space="preserve">Shizuoka</t>
@@ -267,7 +273,7 @@
     <t xml:space="preserve">28 Oct – 2 Nov</t>
   </si>
   <si>
-    <t xml:space="preserve">Day-trip base: Magome–Tsumago walk, Inuyama, Gujo Hachiman, Ise. Transport incl. Shizuoka → Nagoya</t>
+    <t xml:space="preserve">Day-trip base: Magome–Tsumago walk, Inuyama, Gujo Hachiman, Ise. Trains: Shizuoka → Nagoya shinkansen (~£26).</t>
   </si>
   <si>
     <t xml:space="preserve">Takayama</t>
@@ -276,7 +282,7 @@
     <t xml:space="preserve">2 – 5 Nov</t>
   </si>
   <si>
-    <t xml:space="preserve">Peak autumn colour + Culture Day 3 Nov. Shirakawa-go day trip. Transport incl. Nagoya → Takayama</t>
+    <t xml:space="preserve">Peak autumn colour + Culture Day 3 Nov. Shirakawa-go day trip. Trains: Nagoya → Takayama limited express (~£31).</t>
   </si>
   <si>
     <t xml:space="preserve">Osaka (stay in Namba)</t>
@@ -321,7 +327,7 @@
     <t xml:space="preserve">23 – 26 Nov</t>
   </si>
   <si>
-    <t xml:space="preserve">Food capital. Transport incl. HSR from Taipei + Kaohsiung airport for 26 Nov flight</t>
+    <t xml:space="preserve">Food capital. Local transport incl. getting to Kaohsiung airport for the 26 Nov flight. Trains: Taipei → Tainan high-speed rail (~£33).</t>
   </si>
   <si>
     <t xml:space="preserve">Kuala Lumpur</t>
@@ -399,7 +405,7 @@
     <t xml:space="preserve">16 – 18 Jan</t>
   </si>
   <si>
-    <t xml:space="preserve">Transport incl. Hakodate → Tokyo shinkansen. Flight home 08:30 on 18 Jan</t>
+    <t xml:space="preserve">Flight home 08:30 on 18 Jan. Trains: Hakodate → Tokyo shinkansen (~£118).</t>
   </si>
   <si>
     <t xml:space="preserve">Hotels &amp; stays – one row per stop</t>
@@ -1081,13 +1087,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\£#,##0;&quot;(£&quot;#,##0\);\-"/>
-    <numFmt numFmtId="166" formatCode="General"/>
-    <numFmt numFmtId="167" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="168" formatCode="0.0%"/>
-    <numFmt numFmtId="169" formatCode="ddd\ d\ mmm\ yyyy"/>
+    <numFmt numFmtId="166" formatCode="\£#,##0.00;&quot;(£&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="ddd\ d\ mmm\ yyyy"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -1314,7 +1319,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1346,7 +1351,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1354,15 +1363,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1370,7 +1379,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1378,19 +1387,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1418,11 +1423,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1466,19 +1471,19 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1486,7 +1491,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1579,34 +1584,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1751,8 +1756,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="36"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
@@ -2141,19 +2146,19 @@
       </c>
       <c r="B23" s="17" t="n">
         <f aca="false">Itinerary!G25</f>
-        <v>970</v>
+        <v>739</v>
       </c>
       <c r="C23" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A23)</f>
-        <v>32.1</v>
+        <v>8.85</v>
       </c>
       <c r="D23" s="18" t="n">
         <f aca="false">B23-C23</f>
-        <v>937.9</v>
+        <v>730.15</v>
       </c>
       <c r="E23" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B23/$B$3)</f>
-        <v>0.097</v>
+        <v>0.0739</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2161,20 +2166,20 @@
         <v>37</v>
       </c>
       <c r="B24" s="17" t="n">
-        <f aca="false">Itinerary!H25</f>
-        <v>1030</v>
+        <f aca="false">Itinerary!P25</f>
+        <v>231</v>
       </c>
       <c r="C24" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A24)</f>
-        <v>0</v>
+        <v>23.25</v>
       </c>
       <c r="D24" s="18" t="n">
         <f aca="false">B24-C24</f>
-        <v>1030</v>
+        <v>207.75</v>
       </c>
       <c r="E24" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B24/$B$3)</f>
-        <v>0.103</v>
+        <v>0.0231</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2182,20 +2187,20 @@
         <v>38</v>
       </c>
       <c r="B25" s="17" t="n">
-        <f aca="false">Itinerary!O25</f>
-        <v>455</v>
+        <f aca="false">Itinerary!H25</f>
+        <v>1030</v>
       </c>
       <c r="C25" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A25)</f>
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="D25" s="18" t="n">
         <f aca="false">B25-C25</f>
-        <v>451.6</v>
+        <v>1030</v>
       </c>
       <c r="E25" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B25/$B$3)</f>
-        <v>0.0455</v>
+        <v>0.103</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2203,130 +2208,142 @@
         <v>39</v>
       </c>
       <c r="B26" s="17" t="n">
+        <f aca="false">Itinerary!O25</f>
+        <v>455</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A26)</f>
+        <v>3.4</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <f aca="false">B26-C26</f>
+        <v>451.6</v>
+      </c>
+      <c r="E26" s="19" t="n">
+        <f aca="false">IF($B$3=0,0,B26/$B$3)</f>
+        <v>0.0455</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="B27" s="17" t="n">
         <f aca="false">'Admin &amp; checklist'!B9</f>
         <v>457.66</v>
       </c>
-      <c r="C26" s="18" t="n">
-        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A26)</f>
+      <c r="C27" s="18" t="n">
+        <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A27)</f>
         <v>346.66</v>
       </c>
-      <c r="D26" s="18" t="n">
-        <f aca="false">B26-C26</f>
+      <c r="D27" s="18" t="n">
+        <f aca="false">B27-C27</f>
         <v>111</v>
       </c>
-      <c r="E26" s="19" t="n">
-        <f aca="false">IF($B$3=0,0,B26/$B$3)</f>
+      <c r="E27" s="19" t="n">
+        <f aca="false">IF($B$3=0,0,B27/$B$3)</f>
         <v>0.045766</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="B27" s="21" t="n">
-        <f aca="false">$B$3-SUM(B20:B26)</f>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B28" s="21" t="n">
+        <f aca="false">$B$3-SUM(B20:B27)</f>
         <v>-1774</v>
       </c>
-      <c r="C27" s="22" t="n">
+      <c r="C28" s="22" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,"Other")</f>
         <v>0</v>
       </c>
-      <c r="D27" s="22" t="n">
-        <f aca="false">B27-C27</f>
+      <c r="D28" s="22" t="n">
+        <f aca="false">B28-C28</f>
         <v>-1774</v>
       </c>
-      <c r="E27" s="23" t="n">
-        <f aca="false">IF($B$3=0,0,B27/$B$3)</f>
+      <c r="E28" s="23" t="n">
+        <f aca="false">IF($B$3=0,0,B28/$B$3)</f>
         <v>-0.1774</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="24" t="n">
-        <f aca="false">SUM(B20:B27)</f>
+      <c r="B29" s="24" t="n">
+        <f aca="false">SUM(B20:B28)</f>
         <v>10000</v>
       </c>
-      <c r="C28" s="24" t="n">
-        <f aca="false">SUM(C20:C27)</f>
+      <c r="C29" s="24" t="n">
+        <f aca="false">SUM(C20:C28)</f>
         <v>2805.05</v>
       </c>
-      <c r="D28" s="24" t="n">
-        <f aca="false">SUM(D20:D27)</f>
+      <c r="D29" s="24" t="n">
+        <f aca="false">SUM(D20:D28)</f>
         <v>7194.95</v>
       </c>
-      <c r="E28" s="25" t="n">
-        <f aca="false">SUM(E20:E27)</f>
+      <c r="E29" s="25" t="n">
+        <f aca="false">SUM(E20:E28)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="26" t="str">
-        <f aca="false">IF(B27&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B27,"£#,##0"),IF(B27&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="str">
+        <f aca="false">IF(B28&lt;0,"⚠ Plan is over budget by "&amp;TEXT(-B28,"£#,##0"),IF(B28&lt;200,"⚠ Buffer below £200","✓ Plan fits the budget with a buffer"))</f>
         <v>⚠ Plan is over budget by £1,774</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="s">
-        <v>41</v>
-      </c>
-    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+      <c r="A32" s="6" t="s">
         <v>42</v>
-      </c>
-      <c r="B32" s="27" t="n">
-        <f aca="false">Tracker!I4</f>
-        <v>2805.05</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="22" t="n">
-        <f aca="false">Tracker!I5</f>
-        <v>0</v>
+      <c r="B33" s="27" t="n">
+        <f aca="false">Tracker!I4</f>
+        <v>2805.05</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B34" s="27" t="n">
+      <c r="B34" s="22" t="n">
+        <f aca="false">Tracker!I5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B35" s="27" t="n">
         <f aca="false">Tracker!I7</f>
         <v>7194.95</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
         <v>46</v>
       </c>
     </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20" t="s">
+      <c r="A39" s="6" t="s">
         <v>47</v>
-      </c>
-      <c r="B39" s="28" t="n">
-        <v>8034.27</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="B40" s="27" t="n">
-        <f aca="false">Tracker!I4</f>
-        <v>2805.05</v>
+      <c r="B40" s="28" t="n">
+        <v>8034.27</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2334,8 +2351,8 @@
         <v>49</v>
       </c>
       <c r="B41" s="27" t="n">
-        <f aca="false">B39-B40</f>
-        <v>5229.22</v>
+        <f aca="false">Tracker!I4</f>
+        <v>2805.05</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2343,8 +2360,8 @@
         <v>50</v>
       </c>
       <c r="B42" s="27" t="n">
-        <f aca="false">MAX(0,B3-B39)</f>
-        <v>1965.73</v>
+        <f aca="false">B40-B41</f>
+        <v>5229.22</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2352,7 +2369,16 @@
         <v>51</v>
       </c>
       <c r="B43" s="27" t="n">
-        <f aca="false">MAX(0,SUM(B20:B26)-B39)</f>
+        <f aca="false">MAX(0,B3-B40)</f>
+        <v>1965.73</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B44" s="27" t="n">
+        <f aca="false">MAX(0,SUM(B20:B27)-B40)</f>
         <v>3739.73</v>
       </c>
     </row>
@@ -2372,8 +2398,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O25"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:P25"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
@@ -2386,17 +2412,17 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2404,7 +2430,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="7" t="s">
         <v>5</v>
@@ -2413,37 +2439,40 @@
         <v>6</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="N4" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2451,10 +2480,10 @@
         <v>11</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D5" s="29" t="n">
         <v>1</v>
@@ -2481,7 +2510,7 @@
         <v>15</v>
       </c>
       <c r="K5" s="12" t="n">
-        <f aca="false">G5+H5+I5+J5+O5</f>
+        <f aca="false">G5+H5+I5+J5+O5+P5</f>
         <v>71</v>
       </c>
       <c r="L5" s="12" t="n">
@@ -2493,10 +2522,13 @@
         <v>Yes</v>
       </c>
       <c r="N5" s="31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="O5" s="30" t="n">
         <v>5</v>
+      </c>
+      <c r="P5" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2504,10 +2536,10 @@
         <v>11</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D6" s="29" t="n">
         <v>2</v>
@@ -2534,7 +2566,7 @@
         <v>60</v>
       </c>
       <c r="K6" s="12" t="n">
-        <f aca="false">G6+H6+I6+J6+O6</f>
+        <f aca="false">G6+H6+I6+J6+O6+P6</f>
         <v>125</v>
       </c>
       <c r="L6" s="12" t="n">
@@ -2546,10 +2578,13 @@
         <v>N/A – host</v>
       </c>
       <c r="N6" s="31" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="O6" s="30" t="n">
         <v>10</v>
+      </c>
+      <c r="P6" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2557,10 +2592,10 @@
         <v>13</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D7" s="29" t="n">
         <v>3</v>
@@ -2573,7 +2608,7 @@
         <v>38</v>
       </c>
       <c r="G7" s="30" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="H7" s="30" t="n">
         <v>30</v>
@@ -2587,7 +2622,7 @@
         <v>114</v>
       </c>
       <c r="K7" s="12" t="n">
-        <f aca="false">G7+H7+I7+J7+O7</f>
+        <f aca="false">G7+H7+I7+J7+O7+P7</f>
         <v>490.79</v>
       </c>
       <c r="L7" s="12" t="n">
@@ -2599,10 +2634,13 @@
         <v>Yes</v>
       </c>
       <c r="N7" s="31" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="O7" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P7" s="30" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2610,10 +2648,10 @@
         <v>13</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D8" s="29" t="n">
         <v>3</v>
@@ -2640,7 +2678,7 @@
         <v>114</v>
       </c>
       <c r="K8" s="12" t="n">
-        <f aca="false">G8+H8+I8+J8+O8</f>
+        <f aca="false">G8+H8+I8+J8+O8+P8</f>
         <v>428.04</v>
       </c>
       <c r="L8" s="12" t="n">
@@ -2652,10 +2690,13 @@
         <v>Yes</v>
       </c>
       <c r="N8" s="31" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O8" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P8" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2663,10 +2704,10 @@
         <v>13</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D9" s="29" t="n">
         <v>5</v>
@@ -2679,7 +2720,7 @@
         <v>38</v>
       </c>
       <c r="G9" s="30" t="n">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="H9" s="30" t="n">
         <v>60</v>
@@ -2693,7 +2734,7 @@
         <v>190</v>
       </c>
       <c r="K9" s="12" t="n">
-        <f aca="false">G9+H9+I9+J9+O9</f>
+        <f aca="false">G9+H9+I9+J9+O9+P9</f>
         <v>688.05</v>
       </c>
       <c r="L9" s="12" t="n">
@@ -2705,10 +2746,13 @@
         <v>Yes</v>
       </c>
       <c r="N9" s="31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="O9" s="30" t="n">
         <v>25</v>
+      </c>
+      <c r="P9" s="30" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2716,10 +2760,10 @@
         <v>13</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D10" s="29" t="n">
         <v>3</v>
@@ -2732,7 +2776,7 @@
         <v>38</v>
       </c>
       <c r="G10" s="30" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="H10" s="30" t="n">
         <v>40</v>
@@ -2746,7 +2790,7 @@
         <v>114</v>
       </c>
       <c r="K10" s="12" t="n">
-        <f aca="false">G10+H10+I10+J10+O10</f>
+        <f aca="false">G10+H10+I10+J10+O10+P10</f>
         <v>440.17</v>
       </c>
       <c r="L10" s="12" t="n">
@@ -2758,10 +2802,13 @@
         <v>Yes</v>
       </c>
       <c r="N10" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O10" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P10" s="30" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2769,10 +2816,10 @@
         <v>13</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D11" s="29" t="n">
         <v>6</v>
@@ -2799,7 +2846,7 @@
         <v>348</v>
       </c>
       <c r="K11" s="12" t="n">
-        <f aca="false">G11+H11+I11+J11+O11</f>
+        <f aca="false">G11+H11+I11+J11+O11+P11</f>
         <v>818.97</v>
       </c>
       <c r="L11" s="12" t="n">
@@ -2811,10 +2858,13 @@
         <v>Yes</v>
       </c>
       <c r="N11" s="31" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O11" s="30" t="n">
         <v>30</v>
+      </c>
+      <c r="P11" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2822,10 +2872,10 @@
         <v>15</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D12" s="29" t="n">
         <v>3</v>
@@ -2852,7 +2902,7 @@
         <v>45</v>
       </c>
       <c r="K12" s="12" t="n">
-        <f aca="false">G12+H12+I12+J12+O12</f>
+        <f aca="false">G12+H12+I12+J12+O12+P12</f>
         <v>205</v>
       </c>
       <c r="L12" s="12" t="n">
@@ -2864,10 +2914,13 @@
         <v>No</v>
       </c>
       <c r="N12" s="31" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="O12" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P12" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2875,10 +2928,10 @@
         <v>15</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D13" s="29" t="n">
         <v>4</v>
@@ -2905,7 +2958,7 @@
         <v>108</v>
       </c>
       <c r="K13" s="12" t="n">
-        <f aca="false">G13+H13+I13+J13+O13</f>
+        <f aca="false">G13+H13+I13+J13+O13+P13</f>
         <v>313</v>
       </c>
       <c r="L13" s="12" t="n">
@@ -2917,10 +2970,13 @@
         <v>No</v>
       </c>
       <c r="N13" s="31" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="O13" s="30" t="n">
         <v>20</v>
+      </c>
+      <c r="P13" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2928,10 +2984,10 @@
         <v>17</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D14" s="29" t="n">
         <v>5</v>
@@ -2958,7 +3014,7 @@
         <v>237.5</v>
       </c>
       <c r="K14" s="12" t="n">
-        <f aca="false">G14+H14+I14+J14+O14</f>
+        <f aca="false">G14+H14+I14+J14+O14+P14</f>
         <v>557.5</v>
       </c>
       <c r="L14" s="12" t="n">
@@ -2970,10 +3026,13 @@
         <v>No</v>
       </c>
       <c r="N14" s="31" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="O14" s="30" t="n">
         <v>25</v>
+      </c>
+      <c r="P14" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2981,10 +3040,10 @@
         <v>17</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D15" s="29" t="n">
         <v>3</v>
@@ -2997,7 +3056,7 @@
         <v>25</v>
       </c>
       <c r="G15" s="30" t="n">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="H15" s="30" t="n">
         <v>30</v>
@@ -3011,7 +3070,7 @@
         <v>75</v>
       </c>
       <c r="K15" s="12" t="n">
-        <f aca="false">G15+H15+I15+J15+O15</f>
+        <f aca="false">G15+H15+I15+J15+O15+P15</f>
         <v>275</v>
       </c>
       <c r="L15" s="12" t="n">
@@ -3023,10 +3082,13 @@
         <v>No</v>
       </c>
       <c r="N15" s="31" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="O15" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P15" s="30" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3034,10 +3096,10 @@
         <v>19</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D16" s="29" t="n">
         <v>4</v>
@@ -3064,7 +3126,7 @@
         <v>88</v>
       </c>
       <c r="K16" s="12" t="n">
-        <f aca="false">G16+H16+I16+J16+O16</f>
+        <f aca="false">G16+H16+I16+J16+O16+P16</f>
         <v>308</v>
       </c>
       <c r="L16" s="12" t="n">
@@ -3076,10 +3138,13 @@
         <v>No</v>
       </c>
       <c r="N16" s="31" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="O16" s="30" t="n">
         <v>20</v>
+      </c>
+      <c r="P16" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3087,10 +3152,10 @@
         <v>19</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D17" s="29" t="n">
         <v>5</v>
@@ -3117,7 +3182,7 @@
         <v>200</v>
       </c>
       <c r="K17" s="12" t="n">
-        <f aca="false">G17+H17+I17+J17+O17</f>
+        <f aca="false">G17+H17+I17+J17+O17+P17</f>
         <v>490</v>
       </c>
       <c r="L17" s="12" t="n">
@@ -3129,10 +3194,13 @@
         <v>No</v>
       </c>
       <c r="N17" s="31" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="O17" s="30" t="n">
         <v>25</v>
+      </c>
+      <c r="P17" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3140,10 +3208,10 @@
         <v>21</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D18" s="29" t="n">
         <v>5</v>
@@ -3170,7 +3238,7 @@
         <v>225</v>
       </c>
       <c r="K18" s="12" t="n">
-        <f aca="false">G18+H18+I18+J18+O18</f>
+        <f aca="false">G18+H18+I18+J18+O18+P18</f>
         <v>780</v>
       </c>
       <c r="L18" s="12" t="n">
@@ -3182,10 +3250,13 @@
         <v>No</v>
       </c>
       <c r="N18" s="31" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="O18" s="30" t="n">
         <v>25</v>
+      </c>
+      <c r="P18" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3193,10 +3264,10 @@
         <v>21</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D19" s="29" t="n">
         <v>4</v>
@@ -3223,7 +3294,7 @@
         <v>80</v>
       </c>
       <c r="K19" s="12" t="n">
-        <f aca="false">G19+H19+I19+J19+O19</f>
+        <f aca="false">G19+H19+I19+J19+O19+P19</f>
         <v>325</v>
       </c>
       <c r="L19" s="12" t="n">
@@ -3235,10 +3306,13 @@
         <v>No</v>
       </c>
       <c r="N19" s="31" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="O19" s="30" t="n">
         <v>20</v>
+      </c>
+      <c r="P19" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3246,7 +3320,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>23</v>
@@ -3276,7 +3350,7 @@
         <v>760</v>
       </c>
       <c r="K20" s="12" t="n">
-        <f aca="false">G20+H20+I20+J20+O20</f>
+        <f aca="false">G20+H20+I20+J20+O20+P20</f>
         <v>1140</v>
       </c>
       <c r="L20" s="12" t="n">
@@ -3288,10 +3362,13 @@
         <v>N/A – host</v>
       </c>
       <c r="N20" s="31" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="O20" s="30" t="n">
         <v>100</v>
+      </c>
+      <c r="P20" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3299,10 +3376,10 @@
         <v>13</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D21" s="29" t="n">
         <v>8</v>
@@ -3329,7 +3406,7 @@
         <v>384</v>
       </c>
       <c r="K21" s="12" t="n">
-        <f aca="false">G21+H21+I21+J21+O21</f>
+        <f aca="false">G21+H21+I21+J21+O21+P21</f>
         <v>1034</v>
       </c>
       <c r="L21" s="12" t="n">
@@ -3341,10 +3418,13 @@
         <v>No</v>
       </c>
       <c r="N21" s="31" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="O21" s="30" t="n">
         <v>40</v>
+      </c>
+      <c r="P21" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3352,10 +3432,10 @@
         <v>13</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D22" s="29" t="n">
         <v>2</v>
@@ -3382,7 +3462,7 @@
         <v>40</v>
       </c>
       <c r="K22" s="12" t="n">
-        <f aca="false">G22+H22+I22+J22+O22</f>
+        <f aca="false">G22+H22+I22+J22+O22+P22</f>
         <v>360</v>
       </c>
       <c r="L22" s="12" t="n">
@@ -3394,10 +3474,13 @@
         <v>No</v>
       </c>
       <c r="N22" s="31" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="O22" s="30" t="n">
         <v>10</v>
+      </c>
+      <c r="P22" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3405,10 +3488,10 @@
         <v>13</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D23" s="29" t="n">
         <v>3</v>
@@ -3435,7 +3518,7 @@
         <v>114</v>
       </c>
       <c r="K23" s="12" t="n">
-        <f aca="false">G23+H23+I23+J23+O23</f>
+        <f aca="false">G23+H23+I23+J23+O23+P23</f>
         <v>354</v>
       </c>
       <c r="L23" s="12" t="n">
@@ -3447,10 +3530,13 @@
         <v>No</v>
       </c>
       <c r="N23" s="31" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="O23" s="30" t="n">
         <v>15</v>
+      </c>
+      <c r="P23" s="30" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3458,10 +3544,10 @@
         <v>13</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D24" s="29" t="n">
         <v>2</v>
@@ -3474,7 +3560,7 @@
         <v>38</v>
       </c>
       <c r="G24" s="30" t="n">
-        <v>130</v>
+        <v>12</v>
       </c>
       <c r="H24" s="30" t="n">
         <v>30</v>
@@ -3488,7 +3574,7 @@
         <v>76</v>
       </c>
       <c r="K24" s="12" t="n">
-        <f aca="false">G24+H24+I24+J24+O24</f>
+        <f aca="false">G24+H24+I24+J24+O24+P24</f>
         <v>406</v>
       </c>
       <c r="L24" s="12" t="n">
@@ -3500,10 +3586,13 @@
         <v>No</v>
       </c>
       <c r="N24" s="31" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="O24" s="30" t="n">
         <v>10</v>
+      </c>
+      <c r="P24" s="30" t="n">
+        <v>118</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3520,7 +3609,7 @@
       <c r="F25" s="15"/>
       <c r="G25" s="16" t="n">
         <f aca="false">SUM(G5:G24)</f>
-        <v>970</v>
+        <v>739</v>
       </c>
       <c r="H25" s="16" t="n">
         <f aca="false">SUM(H5:H24)</f>
@@ -3547,6 +3636,10 @@
       <c r="O25" s="16" t="n">
         <f aca="false">SUM(O5:O24)</f>
         <v>455</v>
+      </c>
+      <c r="P25" s="16" t="n">
+        <f aca="false">SUM(P5:P24)</f>
+        <v>231</v>
       </c>
     </row>
   </sheetData>
@@ -3566,7 +3659,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N29"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
@@ -3586,12 +3679,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3599,43 +3692,43 @@
         <v>4</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D4" s="33" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J4" s="33" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="K4" s="33" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="L4" s="33" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="M4" s="33" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="N4" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3659,10 +3752,10 @@
         <v>46315</v>
       </c>
       <c r="F5" s="37" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H5" s="39" t="n">
         <v>36</v>
@@ -3672,17 +3765,17 @@
         <v>36</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K5" s="37"/>
       <c r="L5" s="37" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="N5" s="41" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3707,10 +3800,10 @@
         <v>46317</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H6" s="39" t="n">
         <v>0</v>
@@ -3720,13 +3813,13 @@
         <v>0</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="K6" s="37"/>
       <c r="L6" s="37"/>
       <c r="M6" s="37"/>
       <c r="N6" s="41" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3751,10 +3844,10 @@
         <v>46320</v>
       </c>
       <c r="F7" s="37" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H7" s="39" t="n">
         <f aca="false">(52.24+239.55)/3</f>
@@ -3765,13 +3858,13 @@
         <v>291.79</v>
       </c>
       <c r="J7" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K7" s="37"/>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
       <c r="N7" s="41" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3796,10 +3889,10 @@
         <v>46323</v>
       </c>
       <c r="F8" s="37" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H8" s="39" t="n">
         <f aca="false">(137.26+66.78)/3</f>
@@ -3810,13 +3903,13 @@
         <v>204.04</v>
       </c>
       <c r="J8" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K8" s="37"/>
       <c r="L8" s="37"/>
       <c r="M8" s="37"/>
       <c r="N8" s="41" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3841,10 +3934,10 @@
         <v>46328</v>
       </c>
       <c r="F9" s="37" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G9" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H9" s="39" t="n">
         <f aca="false">338.05/5</f>
@@ -3855,13 +3948,13 @@
         <v>338.05</v>
       </c>
       <c r="J9" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K9" s="37"/>
       <c r="L9" s="37"/>
       <c r="M9" s="37"/>
       <c r="N9" s="41" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3886,10 +3979,10 @@
         <v>46331</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H10" s="39" t="n">
         <f aca="false">226.17/3</f>
@@ -3900,13 +3993,13 @@
         <v>226.17</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K10" s="37"/>
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
       <c r="N10" s="41" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3931,10 +4024,10 @@
         <v>46337</v>
       </c>
       <c r="F11" s="37" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G11" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H11" s="39" t="n">
         <f aca="false">300.97/6</f>
@@ -3945,13 +4038,13 @@
         <v>300.97</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K11" s="37"/>
       <c r="L11" s="37"/>
       <c r="M11" s="37"/>
       <c r="N11" s="41" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3977,7 +4070,7 @@
       </c>
       <c r="F12" s="37"/>
       <c r="G12" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H12" s="39" t="n">
         <v>20</v>
@@ -3991,7 +4084,7 @@
       <c r="L12" s="37"/>
       <c r="M12" s="37"/>
       <c r="N12" s="41" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4017,7 +4110,7 @@
       </c>
       <c r="F13" s="37"/>
       <c r="G13" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H13" s="39" t="n">
         <v>25</v>
@@ -4031,7 +4124,7 @@
       <c r="L13" s="37"/>
       <c r="M13" s="37"/>
       <c r="N13" s="41" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4057,7 +4150,7 @@
       </c>
       <c r="F14" s="37"/>
       <c r="G14" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H14" s="39" t="n">
         <v>45</v>
@@ -4095,7 +4188,7 @@
       </c>
       <c r="F15" s="37"/>
       <c r="G15" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H15" s="39" t="n">
         <v>35</v>
@@ -4133,7 +4226,7 @@
       </c>
       <c r="F16" s="37"/>
       <c r="G16" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H16" s="39" t="n">
         <v>35</v>
@@ -4171,7 +4264,7 @@
       </c>
       <c r="F17" s="37"/>
       <c r="G17" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H17" s="39" t="n">
         <v>25</v>
@@ -4185,7 +4278,7 @@
       <c r="L17" s="37"/>
       <c r="M17" s="37"/>
       <c r="N17" s="41" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4211,7 +4304,7 @@
       </c>
       <c r="F18" s="37"/>
       <c r="G18" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H18" s="39" t="n">
         <v>90</v>
@@ -4225,7 +4318,7 @@
       <c r="L18" s="37"/>
       <c r="M18" s="37"/>
       <c r="N18" s="41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4251,7 +4344,7 @@
       </c>
       <c r="F19" s="37"/>
       <c r="G19" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H19" s="39" t="n">
         <v>35</v>
@@ -4288,10 +4381,10 @@
         <v>46390</v>
       </c>
       <c r="F20" s="37" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G20" s="38" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H20" s="39" t="n">
         <v>0</v>
@@ -4301,13 +4394,13 @@
         <v>0</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="K20" s="37"/>
       <c r="L20" s="37"/>
       <c r="M20" s="37"/>
       <c r="N20" s="41" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4333,7 +4426,7 @@
       </c>
       <c r="F21" s="37"/>
       <c r="G21" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H21" s="39" t="n">
         <v>55</v>
@@ -4347,7 +4440,7 @@
       <c r="L21" s="37"/>
       <c r="M21" s="37"/>
       <c r="N21" s="41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4373,7 +4466,7 @@
       </c>
       <c r="F22" s="37"/>
       <c r="G22" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H22" s="39" t="n">
         <v>130</v>
@@ -4387,7 +4480,7 @@
       <c r="L22" s="37"/>
       <c r="M22" s="37"/>
       <c r="N22" s="41" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4413,7 +4506,7 @@
       </c>
       <c r="F23" s="37"/>
       <c r="G23" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H23" s="39" t="n">
         <v>55</v>
@@ -4451,7 +4544,7 @@
       </c>
       <c r="F24" s="37"/>
       <c r="G24" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H24" s="39" t="n">
         <v>80</v>
@@ -4465,7 +4558,7 @@
       <c r="L24" s="37"/>
       <c r="M24" s="37"/>
       <c r="N24" s="41" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4498,7 +4591,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C27" s="44" t="str">
         <f aca="false">COUNTIF(G5:G24,"Booked")&amp;" of "&amp;(COUNTA(G5:G24)-COUNTIF(G5:G24,"Staying with friends"))</f>
@@ -4507,7 +4600,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C28" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"Booked",I5:I24)</f>
@@ -4516,7 +4609,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C29" s="45" t="n">
         <f aca="false">SUMIF(G5:G24,"To book",I5:I24)+SUMIF(G5:G24,"Shortlisted",I5:I24)</f>
@@ -4555,7 +4648,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M21"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17"/>
@@ -4571,53 +4664,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="32" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="33" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B4" s="33" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C4" s="33" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F4" s="33" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="G4" s="33" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H4" s="33" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="I4" s="33" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J4" s="33" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="K4" s="33" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="L4" s="33" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="M4" s="33" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4628,33 +4721,33 @@
         <v>46313</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E5" s="38" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F5" s="38" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="G5" s="38"/>
       <c r="H5" s="38" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I5" s="47" t="n">
         <v>667.6</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K5" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L5" s="38"/>
       <c r="M5" s="41" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4665,35 +4758,35 @@
         <v>46314</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E6" s="38" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H6" s="38" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I6" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K6" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L6" s="38"/>
       <c r="M6" s="41" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4704,35 +4797,35 @@
         <v>46317</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="E7" s="38" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F7" s="38" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="G7" s="38" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H7" s="38" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="I7" s="47" t="n">
         <v>87.7</v>
       </c>
       <c r="J7" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K7" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L7" s="38"/>
       <c r="M7" s="41" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4743,35 +4836,35 @@
         <v>46337</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E8" s="38" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F8" s="38" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="G8" s="38" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="H8" s="38" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="I8" s="47" t="n">
         <v>211.52</v>
       </c>
       <c r="J8" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K8" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L8" s="38"/>
       <c r="M8" s="41" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4782,29 +4875,29 @@
         <v>46344</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="E9" s="38"/>
       <c r="F9" s="38"/>
       <c r="G9" s="38"/>
       <c r="H9" s="38" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="I9" s="47" t="n">
         <v>130</v>
       </c>
       <c r="J9" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K9" s="38" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="L9" s="38"/>
       <c r="M9" s="41" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4815,29 +4908,29 @@
         <v>46352</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D10" s="38" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="E10" s="38"/>
       <c r="F10" s="38"/>
       <c r="G10" s="38"/>
       <c r="H10" s="38" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="I10" s="47" t="n">
         <v>130</v>
       </c>
       <c r="J10" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L10" s="38"/>
       <c r="M10" s="41" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4848,29 +4941,29 @@
         <v>46361</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D11" s="38" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E11" s="38"/>
       <c r="F11" s="38"/>
       <c r="G11" s="38"/>
       <c r="H11" s="38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I11" s="47" t="n">
         <v>80</v>
       </c>
       <c r="J11" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K11" s="38" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L11" s="38"/>
       <c r="M11" s="41" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4881,29 +4974,29 @@
         <v>46366</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="E12" s="38"/>
       <c r="F12" s="38"/>
       <c r="G12" s="38"/>
       <c r="H12" s="38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I12" s="47" t="n">
         <v>70</v>
       </c>
       <c r="J12" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="L12" s="38"/>
       <c r="M12" s="41" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4914,29 +5007,29 @@
         <v>46370</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E13" s="38"/>
       <c r="F13" s="38"/>
       <c r="G13" s="38"/>
       <c r="H13" s="38" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="I13" s="47" t="n">
         <v>180</v>
       </c>
       <c r="J13" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K13" s="38" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="L13" s="38"/>
       <c r="M13" s="41" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4947,29 +5040,29 @@
         <v>46390</v>
       </c>
       <c r="C14" s="38" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="E14" s="38"/>
       <c r="F14" s="38"/>
       <c r="G14" s="38"/>
       <c r="H14" s="38" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I14" s="47" t="n">
         <v>150</v>
       </c>
       <c r="J14" s="38" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="L14" s="38"/>
       <c r="M14" s="41" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4980,31 +5073,31 @@
         <v>46405</v>
       </c>
       <c r="C15" s="38" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E15" s="38" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F15" s="38" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G15" s="38" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="H15" s="38" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I15" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K15" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L15" s="38"/>
       <c r="M15" s="41"/>
@@ -5017,35 +5110,35 @@
         <v>46405</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F16" s="38" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="I16" s="47" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="38" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="L16" s="38"/>
       <c r="M16" s="41" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5070,7 +5163,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I18" s="49" t="n">
         <f aca="false">SUMIF(J5:J16,"Booked",I5:I16)</f>
@@ -5079,7 +5172,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="I19" s="49" t="n">
         <f aca="false">I17-I18</f>
@@ -5088,7 +5181,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="32" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
   </sheetData>
@@ -5119,7 +5212,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="60"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
@@ -5129,82 +5222,82 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B5" s="28" t="n">
         <v>281.62</v>
       </c>
       <c r="C5" s="29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D5" s="31" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B6" s="28" t="n">
         <v>62.4</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D6" s="31" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B7" s="28" t="n">
         <v>13.64</v>
       </c>
       <c r="C7" s="29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B8" s="28" t="n">
         <v>100</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D8" s="31" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5220,225 +5313,225 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="8" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C13" s="29"/>
       <c r="D13" s="31"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="8" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C14" s="29"/>
       <c r="D14" s="31"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C15" s="29"/>
       <c r="D15" s="31" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C16" s="29"/>
       <c r="D16" s="31" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="8" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C17" s="29"/>
       <c r="D17" s="31" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C18" s="29"/>
       <c r="D18" s="31"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="8" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C19" s="29"/>
       <c r="D19" s="31" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="8" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C20" s="29"/>
       <c r="D20" s="31" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C21" s="29"/>
       <c r="D21" s="31" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C22" s="29"/>
       <c r="D22" s="31"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="8" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C23" s="29"/>
       <c r="D23" s="31"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C24" s="29"/>
       <c r="D24" s="31" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="8" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C25" s="29"/>
       <c r="D25" s="31" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="8" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C26" s="29"/>
       <c r="D26" s="31"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C27" s="29"/>
       <c r="D27" s="31"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="8" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C28" s="29"/>
       <c r="D28" s="31"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="8" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C29" s="29"/>
       <c r="D29" s="31"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="8" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C30" s="29"/>
       <c r="D30" s="31"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="8" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C31" s="29"/>
       <c r="D31" s="31"/>
@@ -5480,7 +5573,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="20"/>
@@ -5496,17 +5589,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B4" s="7" t="s">
         <v>4</v>
@@ -5515,46 +5608,46 @@
         <v>30</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
         <v>2805.05</v>
       </c>
       <c r="J4" s="7" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B5" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C5" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D5" s="51" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E5" s="52" t="n">
         <v>667.6</v>
       </c>
       <c r="F5" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H5" s="20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I5" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Booked – pay later")</f>
@@ -5563,25 +5656,25 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B6" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C6" s="51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D6" s="51" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="E6" s="52" t="n">
         <v>281.62</v>
       </c>
       <c r="F6" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
@@ -5590,7 +5683,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B7" s="51" t="s">
         <v>11</v>
@@ -5599,16 +5692,16 @@
         <v>34</v>
       </c>
       <c r="D7" s="51" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="E7" s="52" t="n">
         <v>36</v>
       </c>
       <c r="F7" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H7" s="20" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
@@ -5617,47 +5710,47 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B8" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C8" s="51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D8" s="51" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="E8" s="52" t="n">
         <v>19</v>
       </c>
       <c r="F8" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B9" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C9" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D9" s="51" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E9" s="52" t="n">
         <v>87.7</v>
       </c>
       <c r="F9" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B10" s="51" t="s">
         <v>13</v>
@@ -5666,18 +5759,18 @@
         <v>34</v>
       </c>
       <c r="D10" s="51" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="E10" s="52" t="n">
         <v>239.55</v>
       </c>
       <c r="F10" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B11" s="51" t="s">
         <v>13</v>
@@ -5686,38 +5779,38 @@
         <v>34</v>
       </c>
       <c r="D11" s="51" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="E11" s="52" t="n">
         <v>52.24</v>
       </c>
       <c r="F11" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B12" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C12" s="51" t="s">
         <v>33</v>
       </c>
       <c r="D12" s="51" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="E12" s="52" t="n">
         <v>211.52</v>
       </c>
       <c r="F12" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="51" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B13" s="51" t="s">
         <v>13</v>
@@ -5726,18 +5819,18 @@
         <v>34</v>
       </c>
       <c r="D13" s="51" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E13" s="52" t="n">
         <v>137.26</v>
       </c>
       <c r="F13" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="51" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B14" s="51" t="s">
         <v>13</v>
@@ -5746,18 +5839,18 @@
         <v>34</v>
       </c>
       <c r="D14" s="51" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E14" s="52" t="n">
         <v>338.05</v>
       </c>
       <c r="F14" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B15" s="51" t="s">
         <v>13</v>
@@ -5766,18 +5859,18 @@
         <v>34</v>
       </c>
       <c r="D15" s="51" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E15" s="52" t="n">
         <v>66.78</v>
       </c>
       <c r="F15" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B16" s="51" t="s">
         <v>13</v>
@@ -5786,18 +5879,18 @@
         <v>34</v>
       </c>
       <c r="D16" s="51" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="E16" s="52" t="n">
         <v>300.97</v>
       </c>
       <c r="F16" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="51" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B17" s="51" t="s">
         <v>13</v>
@@ -5806,58 +5899,58 @@
         <v>34</v>
       </c>
       <c r="D17" s="51" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="E17" s="52" t="n">
         <v>226.17</v>
       </c>
       <c r="F17" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="51" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B18" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C18" s="51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D18" s="51" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E18" s="52" t="n">
         <v>13.64</v>
       </c>
       <c r="F18" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="51" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B19" s="51" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C19" s="51" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D19" s="51" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="E19" s="52" t="n">
         <v>32.4</v>
       </c>
       <c r="F19" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="51" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B20" s="51" t="s">
         <v>11</v>
@@ -5866,21 +5959,21 @@
         <v>36</v>
       </c>
       <c r="D20" s="51" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E20" s="52" t="n">
         <v>2.95</v>
       </c>
       <c r="F20" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="51" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B21" s="51" t="s">
         <v>11</v>
@@ -5889,21 +5982,21 @@
         <v>35</v>
       </c>
       <c r="D21" s="51" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E21" s="52" t="n">
         <v>3.05</v>
       </c>
       <c r="F21" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="51" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B22" s="51" t="s">
         <v>11</v>
@@ -5918,15 +6011,15 @@
         <v>14.91</v>
       </c>
       <c r="F22" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B23" s="51" t="s">
         <v>11</v>
@@ -5935,21 +6028,21 @@
         <v>35</v>
       </c>
       <c r="D23" s="51" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E23" s="52" t="n">
         <v>3.4</v>
       </c>
       <c r="F23" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B24" s="51" t="s">
         <v>11</v>
@@ -5958,21 +6051,21 @@
         <v>35</v>
       </c>
       <c r="D24" s="51" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="E24" s="52" t="n">
         <v>2.55</v>
       </c>
       <c r="F24" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B25" s="51" t="s">
         <v>11</v>
@@ -5981,21 +6074,21 @@
         <v>36</v>
       </c>
       <c r="D25" s="51" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E25" s="52" t="n">
         <v>5.9</v>
       </c>
       <c r="F25" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B26" s="51" t="s">
         <v>11</v>
@@ -6004,21 +6097,21 @@
         <v>35</v>
       </c>
       <c r="D26" s="51" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E26" s="52" t="n">
         <v>8.5</v>
       </c>
       <c r="F26" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B27" s="51" t="s">
         <v>11</v>
@@ -6027,44 +6120,44 @@
         <v>35</v>
       </c>
       <c r="D27" s="51" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E27" s="52" t="n">
         <v>8.87</v>
       </c>
       <c r="F27" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B28" s="51" t="s">
         <v>11</v>
       </c>
       <c r="C28" s="51" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D28" s="51" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="E28" s="52" t="n">
         <v>3.4</v>
       </c>
       <c r="F28" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="51" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B29" s="51" t="s">
         <v>11</v>
@@ -6073,21 +6166,21 @@
         <v>35</v>
       </c>
       <c r="D29" s="51" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E29" s="52" t="n">
         <v>1.98</v>
       </c>
       <c r="F29" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="51" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B30" s="51" t="s">
         <v>11</v>
@@ -6096,44 +6189,44 @@
         <v>35</v>
       </c>
       <c r="D30" s="51" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="E30" s="52" t="n">
         <v>4.26</v>
       </c>
       <c r="F30" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="51" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B31" s="51" t="s">
         <v>13</v>
       </c>
       <c r="C31" s="51" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D31" s="51" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E31" s="52" t="n">
         <v>23.25</v>
       </c>
       <c r="F31" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="51" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B32" s="51" t="s">
         <v>11</v>
@@ -6142,21 +6235,21 @@
         <v>35</v>
       </c>
       <c r="D32" s="51" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="E32" s="52" t="n">
         <v>6.76</v>
       </c>
       <c r="F32" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="51" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B33" s="51" t="s">
         <v>11</v>
@@ -6165,21 +6258,21 @@
         <v>35</v>
       </c>
       <c r="D33" s="51" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E33" s="52" t="n">
         <v>1.99</v>
       </c>
       <c r="F33" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="51" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B34" s="51" t="s">
         <v>11</v>
@@ -6188,16 +6281,16 @@
         <v>35</v>
       </c>
       <c r="D34" s="51" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="E34" s="52" t="n">
         <v>2.78</v>
       </c>
       <c r="F34" s="51" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -13921,7 +14014,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C5:C1000" type="list">
-      <formula1>"Flights,Accommodation,Food,Local transport,Activities,Shopping &amp; misc,Insurance &amp; admin,Other"</formula1>
+      <formula1>"Flights,Accommodation,Food,Local transport,Trains &amp; intercity,Activities,Shopping &amp; misc,Insurance &amp; admin,Other"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F5:F1000" type="list">

</xml_diff>

<commit_message>
Sync Tracker with spend log (0 added, 1 updated, 0 removed)
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -1848,11 +1848,11 @@
       </c>
       <c r="F7" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Korea",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>157.5</v>
+        <v>161.28</v>
       </c>
       <c r="G7" s="12" t="n">
         <f aca="false">D7+D13-F7</f>
-        <v>1178.5</v>
+        <v>1174.72</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2226,11 +2226,11 @@
       </c>
       <c r="C26" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A26)</f>
-        <v>16.97</v>
+        <v>20.75</v>
       </c>
       <c r="D26" s="18" t="n">
         <f aca="false">B26-C26</f>
-        <v>438.03</v>
+        <v>434.25</v>
       </c>
       <c r="E26" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B26/$B$3)</f>
@@ -2289,11 +2289,11 @@
       </c>
       <c r="C29" s="24" t="n">
         <f aca="false">SUM(C20:C28)</f>
-        <v>2855.25</v>
+        <v>2859.03</v>
       </c>
       <c r="D29" s="24" t="n">
         <f aca="false">SUM(D20:D28)</f>
-        <v>7144.75</v>
+        <v>7140.97</v>
       </c>
       <c r="E29" s="25" t="n">
         <f aca="false">SUM(E20:E28)</f>
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2855.25</v>
+        <v>2859.03</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="B35" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7144.75</v>
+        <v>7140.97</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2365,7 +2365,7 @@
       </c>
       <c r="B41" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2855.25</v>
+        <v>2859.03</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2374,7 +2374,7 @@
       </c>
       <c r="B42" s="27" t="n">
         <f aca="false">B40-B41</f>
-        <v>5179.02</v>
+        <v>5175.24</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2855.25</v>
+        <v>2859.03</v>
       </c>
       <c r="J4" s="7" t="s">
         <v>295</v>
@@ -5691,7 +5691,7 @@
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2855.25</v>
+        <v>2859.03</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5718,7 +5718,7 @@
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7144.75</v>
+        <v>7140.97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6343,7 +6343,7 @@
         <v>354</v>
       </c>
       <c r="E36" s="52" t="n">
-        <v>13.57</v>
+        <v>17.35</v>
       </c>
       <c r="F36" s="51" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
Sync Tracker with spend log (0 added, 0 updated, 1 removed)
</commit_message>
<xml_diff>
--- a/Sabbatical_Plan_and_Budget.xlsx
+++ b/Sabbatical_Plan_and_Budget.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="382">
   <si>
     <t xml:space="preserve">Sabbatical 2026–27: plan &amp; budget</t>
   </si>
@@ -1171,12 +1171,6 @@
   </si>
   <si>
     <t xml:space="preserve">mvkj13sckg46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">mvkj2i74n90g</t>
   </si>
 </sst>
 </file>
@@ -1960,11 +1954,11 @@
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Flights")-SUMIFS(Tracker!$E$5:$E$1000,Tracker!$B$5:$B$1000,"Japan",Tracker!$C$5:$C$1000,"Insurance &amp; admin")</f>
-        <v>1509.05</v>
+        <v>1499.05</v>
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">D8+D14-F8</f>
-        <v>3510.97</v>
+        <v>3520.97</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2226,11 +2220,11 @@
       </c>
       <c r="C22" s="18" t="n">
         <f aca="false">SUMIFS(Tracker!$E$5:$E$1000,Tracker!$C$5:$C$1000,A22)</f>
-        <v>178.48</v>
+        <v>168.48</v>
       </c>
       <c r="D22" s="18" t="n">
         <f aca="false">B22-C22</f>
-        <v>3209.02</v>
+        <v>3219.02</v>
       </c>
       <c r="E22" s="19" t="n">
         <f aca="false">IF($B$3=0,0,B22/$B$3)</f>
@@ -2373,11 +2367,11 @@
       </c>
       <c r="C29" s="24" t="n">
         <f aca="false">SUM(C20:C28)</f>
-        <v>2997.38</v>
+        <v>2987.38</v>
       </c>
       <c r="D29" s="24" t="n">
         <f aca="false">SUM(D20:D28)</f>
-        <v>7002.62</v>
+        <v>7012.62</v>
       </c>
       <c r="E29" s="25" t="n">
         <f aca="false">SUM(E20:E28)</f>
@@ -2402,7 +2396,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2997.38</v>
+        <v>2987.38</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2420,7 +2414,7 @@
       </c>
       <c r="B35" s="27" t="n">
         <f aca="false">Tracker!I7</f>
-        <v>7002.62</v>
+        <v>7012.62</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2449,7 +2443,7 @@
       </c>
       <c r="B41" s="27" t="n">
         <f aca="false">Tracker!I4</f>
-        <v>2997.38</v>
+        <v>2987.38</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2458,7 +2452,7 @@
       </c>
       <c r="B42" s="27" t="n">
         <f aca="false">B40-B41</f>
-        <v>5036.89</v>
+        <v>5046.89</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5718,7 +5712,7 @@
       </c>
       <c r="I4" s="50" t="n">
         <f aca="false">SUMIFS(E5:E1000,F5:F1000,"Paid")</f>
-        <v>2997.38</v>
+        <v>2987.38</v>
       </c>
       <c r="J4" s="7" t="s">
         <v>295</v>
@@ -5775,7 +5769,7 @@
       </c>
       <c r="I6" s="24" t="n">
         <f aca="false">I4+I5</f>
-        <v>2997.38</v>
+        <v>2987.38</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5802,7 +5796,7 @@
       </c>
       <c r="I7" s="27" t="n">
         <f aca="false">Overview!B3-I6</f>
-        <v>7002.62</v>
+        <v>7012.62</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6736,27 +6730,12 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="51" t="s">
-        <v>369</v>
-      </c>
-      <c r="B50" s="51" t="s">
-        <v>13</v>
-      </c>
-      <c r="C50" s="51" t="s">
-        <v>35</v>
-      </c>
-      <c r="D50" s="51" t="s">
-        <v>382</v>
-      </c>
-      <c r="E50" s="52" t="n">
-        <v>10</v>
-      </c>
-      <c r="F50" s="51" t="s">
-        <v>43</v>
-      </c>
-      <c r="J50" s="1" t="s">
-        <v>383</v>
-      </c>
+      <c r="A50" s="51"/>
+      <c r="B50" s="51"/>
+      <c r="C50" s="51"/>
+      <c r="D50" s="51"/>
+      <c r="E50" s="52"/>
+      <c r="F50" s="51"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="51"/>

</xml_diff>